<commit_message>
Record entry prices 2026-09-26
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1267,6 +1267,766 @@
       </c>
       <c r="J21" s="4" t="n">
         <v>426.2999877929688</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>2980</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>証券、商品先物取引業</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>電気・ガス業</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>2436</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>非鉄金属</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>食料品</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>2286</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>75</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>1671</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>436</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>輸送用機器</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>90.7</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>2898</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>4855</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>2152</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>5445</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>東京鐵鋼</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>鉄鋼</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>2067</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>医薬品</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>2399</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>5101</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>横浜ゴム</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>6986</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>1191</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>430.2999877929688</v>
       </c>
     </row>
   </sheetData>
@@ -2798,7 +3558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3321,6 +4081,406 @@
         <v>1682</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>2286</v>
+      </c>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>436</v>
+      </c>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>2980</v>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>2436</v>
+      </c>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>1671</v>
+      </c>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>4855</v>
+      </c>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>2152</v>
+      </c>
+      <c r="E28" s="4" t="n"/>
+      <c r="F28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>2898</v>
+      </c>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>2399</v>
+      </c>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>5101</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>横浜ゴム</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>6986</v>
+      </c>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>5445</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>東京鐵鋼</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>2067</v>
+      </c>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="E39" s="4" t="n"/>
+      <c r="F39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="E40" s="4" t="n"/>
+      <c r="F40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>1191</v>
+      </c>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Performance check 2026-09-19 -> 2026-09-26
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -2040,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2185,34 +2185,34 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>システナ</t>
+          <t>丸大食品</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>440</v>
+        <v>2311</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>440</v>
+        <v>2286</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0</v>
+        <v>-0.01081782778018174</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.0202008916191198</v>
       </c>
     </row>
     <row r="5">
@@ -2230,25 +2230,25 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>440</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.01136363636363636</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.01394399323676342</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="6">
@@ -2257,34 +2257,34 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>3080</v>
+        <v>440</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>3080</v>
+        <v>435</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0</v>
+        <v>-0.01136363636363636</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.01394399323676342</v>
       </c>
     </row>
     <row r="7">
@@ -2293,34 +2293,34 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>3080</v>
+        <v>440</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>3135</v>
+        <v>436</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0.01785714285714286</v>
+        <v>-0.00909090909090909</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.0152767859840158</v>
+        <v>-0.01847397292984715</v>
       </c>
     </row>
     <row r="8">
@@ -2329,12 +2329,12 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -2344,10 +2344,10 @@
         <v>2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>0</v>
@@ -2365,12 +2365,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -2380,19 +2380,19 @@
         <v>5</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>2444</v>
+        <v>3135</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.00741962077493817</v>
+        <v>0.01785714285714286</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.004839263901811112</v>
+        <v>0.0152767859840158</v>
       </c>
     </row>
     <row r="10">
@@ -2401,34 +2401,34 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1700</v>
+        <v>3080</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>1700</v>
+        <v>2980</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>0</v>
+        <v>-0.03246753246753246</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.04185059630647053</v>
       </c>
     </row>
     <row r="11">
@@ -2437,34 +2437,34 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>1700</v>
+        <v>2426</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>1689</v>
+        <v>2426</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.006470588235294118</v>
+        <v>0</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.009050945108421176</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="12">
@@ -2473,34 +2473,34 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>4775</v>
+        <v>2426</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>4775</v>
+        <v>2444</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0</v>
+        <v>0.00741962077493817</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.004839263901811112</v>
       </c>
     </row>
     <row r="13">
@@ -2509,34 +2509,34 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>4775</v>
+        <v>2426</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>4795</v>
+        <v>2436</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.004188481675392671</v>
+        <v>0.004122011541632316</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.001608124802265612</v>
+        <v>-0.005261052297305746</v>
       </c>
     </row>
     <row r="14">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -2560,10 +2560,10 @@
         <v>2</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2163</v>
+        <v>1700</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>2163</v>
+        <v>1700</v>
       </c>
       <c r="H14" s="5" t="n">
         <v>0</v>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -2596,19 +2596,19 @@
         <v>5</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>2163</v>
+        <v>1700</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>2175</v>
+        <v>1689</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0.005547850208044383</v>
+        <v>-0.006470588235294118</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.002967493334917325</v>
+        <v>-0.009050945108421176</v>
       </c>
     </row>
     <row r="16">
@@ -2617,34 +2617,34 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>2915</v>
+        <v>1700</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>2915</v>
+        <v>1671</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0</v>
+        <v>-0.01705882352941177</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.02644188736834983</v>
       </c>
     </row>
     <row r="17">
@@ -2653,34 +2653,34 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>2915</v>
+        <v>4775</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>2920</v>
+        <v>4775</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0.001715265866209262</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>-0.0008650910069177959</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="18">
@@ -2689,34 +2689,34 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2383.5</v>
+        <v>4775</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>2383.5</v>
+        <v>4795</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0</v>
+        <v>0.004188481675392671</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.001608124802265612</v>
       </c>
     </row>
     <row r="19">
@@ -2725,34 +2725,34 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>2383.5</v>
+        <v>4775</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>2370.5</v>
+        <v>4855</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.005454164044472415</v>
+        <v>0.01675392670157068</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>-0.008034520917599472</v>
+        <v>0.00737086286263262</v>
       </c>
     </row>
     <row r="20">
@@ -2761,12 +2761,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -2776,10 +2776,10 @@
         <v>2</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>6825</v>
+        <v>2163</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>6825</v>
+        <v>2163</v>
       </c>
       <c r="H20" s="5" t="n">
         <v>0</v>
@@ -2797,12 +2797,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
@@ -2812,19 +2812,19 @@
         <v>5</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>6825</v>
+        <v>2163</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>6964</v>
+        <v>2175</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0.02036630036630037</v>
+        <v>0.005547850208044383</v>
       </c>
       <c r="I21" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.01778594349317331</v>
+        <v>0.002967493334917325</v>
       </c>
     </row>
     <row r="22">
@@ -2833,34 +2833,34 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>5105</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>ＴＯＹＯ　ＴＩＲＥ</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>3804</v>
+        <v>2163</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>3804</v>
+        <v>2152</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0</v>
+        <v>-0.005085529357374018</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.01446859319631208</v>
       </c>
     </row>
     <row r="23">
@@ -2869,34 +2869,34 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>5105</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ＴＯＹＯ　ＴＩＲＥ</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>3804</v>
+        <v>2915</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>3825</v>
+        <v>2915</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>0.005520504731861199</v>
+        <v>0</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>0.002940147858734141</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="24">
@@ -2905,34 +2905,34 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>2454</v>
+        <v>2915</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>2454</v>
+        <v>2920</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0</v>
+        <v>0.001715265866209262</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.0008650910069177959</v>
       </c>
     </row>
     <row r="25">
@@ -2941,34 +2941,34 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>2454</v>
+        <v>2915</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>2466</v>
+        <v>2898</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>0.004889975550122249</v>
+        <v>-0.005831903945111492</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>0.002309618676995191</v>
+        <v>-0.01521496778404955</v>
       </c>
     </row>
     <row r="26">
@@ -2977,12 +2977,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
@@ -2992,10 +2992,10 @@
         <v>2</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>2060</v>
+        <v>2383.5</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>2060</v>
+        <v>2383.5</v>
       </c>
       <c r="H26" s="5" t="n">
         <v>0</v>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
@@ -3028,19 +3028,19 @@
         <v>5</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>2060</v>
+        <v>2383.5</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>2060</v>
+        <v>2370.5</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>0</v>
+        <v>-0.005454164044472415</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>-0.002580356873127058</v>
+        <v>-0.008034520917599472</v>
       </c>
     </row>
     <row r="28">
@@ -3049,34 +3049,34 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>22795</v>
+        <v>2383.5</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>22795</v>
+        <v>2399</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0</v>
+        <v>0.006503041745332494</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.002880022093605568</v>
       </c>
     </row>
     <row r="29">
@@ -3085,34 +3085,34 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>22795</v>
+        <v>6825</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>23605</v>
+        <v>6825</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>0.03553410835709585</v>
+        <v>0</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.0329537514839688</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="30">
@@ -3121,34 +3121,34 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>723</v>
+        <v>6825</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>723</v>
+        <v>6964</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0</v>
+        <v>0.02036630036630037</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.01778594349317331</v>
       </c>
     </row>
     <row r="31">
@@ -3157,34 +3157,34 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>723</v>
+        <v>6825</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>730</v>
+        <v>6986</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>0.009681881051175657</v>
+        <v>0.02358974358974359</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.007101524178048599</v>
+        <v>0.01420667975080553</v>
       </c>
     </row>
     <row r="32">
@@ -3193,12 +3193,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -3208,10 +3208,10 @@
         <v>2</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>3370</v>
+        <v>3804</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>3370</v>
+        <v>3804</v>
       </c>
       <c r="H32" s="5" t="n">
         <v>0</v>
@@ -3229,12 +3229,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
@@ -3244,19 +3244,19 @@
         <v>5</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3370</v>
+        <v>3804</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>3375</v>
+        <v>3825</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>0.001483679525222552</v>
+        <v>0.005520504731861199</v>
       </c>
       <c r="I33" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>-0.001096677347904506</v>
+        <v>0.002940147858734141</v>
       </c>
     </row>
     <row r="34">
@@ -3265,34 +3265,34 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>842</v>
+        <v>3804</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>842</v>
+        <v>3871</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0</v>
+        <v>0.0176130389064143</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.00822997506747624</v>
       </c>
     </row>
     <row r="35">
@@ -3301,34 +3301,34 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>842</v>
+        <v>2454</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>848</v>
+        <v>2454</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>0.007125890736342043</v>
+        <v>0</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>0.004545533863214985</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="36">
@@ -3337,34 +3337,34 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>1488</v>
+        <v>2454</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>1488</v>
+        <v>2466</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0</v>
+        <v>0.004889975550122249</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.002309618676995191</v>
       </c>
     </row>
     <row r="37">
@@ -3373,34 +3373,34 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>1488</v>
+        <v>2454</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>1494</v>
+        <v>2527</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>0.004032258064516129</v>
+        <v>0.02974735126324368</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.001451901191389071</v>
+        <v>0.02036428742430562</v>
       </c>
     </row>
     <row r="38">
@@ -3409,12 +3409,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
@@ -3424,10 +3424,10 @@
         <v>2</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>1287</v>
+        <v>2060</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>1287</v>
+        <v>2060</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>0</v>
@@ -3445,12 +3445,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
@@ -3460,19 +3460,19 @@
         <v>5</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>1287</v>
+        <v>2060</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>1293</v>
+        <v>2060</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>0.004662004662004662</v>
+        <v>0</v>
       </c>
       <c r="I39" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J39" s="5" t="n">
-        <v>0.002081647788877604</v>
+        <v>-0.002580356873127058</v>
       </c>
     </row>
     <row r="40">
@@ -3481,34 +3481,34 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>8624</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>いちよし証券</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>1686</v>
+        <v>2060</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>1686</v>
+        <v>2067</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0</v>
+        <v>0.003398058252427184</v>
       </c>
       <c r="I40" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.005985005586510878</v>
       </c>
     </row>
     <row r="41">
@@ -3517,34 +3517,754 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>22795</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>22795</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>22795</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>23605</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>0.03553410835709585</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J42" s="5" t="n">
+        <v>0.0329537514839688</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>22795</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>0.007896468523799079</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>-0.001486595315138983</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>723</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>723</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J44" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>723</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>730</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>0.009681881051175657</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>0.007101524178048599</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>723</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>-0.06639004149377593</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J46" s="5" t="n">
+        <v>-0.075773105332714</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J47" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>3375</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>0.001483679525222552</v>
+      </c>
+      <c r="I48" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J48" s="5" t="n">
+        <v>-0.001096677347904506</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>-0.01335311572700297</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J49" s="5" t="n">
+        <v>-0.02273617956594103</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J50" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>848</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>0.007125890736342043</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J51" s="5" t="n">
+        <v>0.004545533863214985</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>0.04513064133016627</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J52" s="5" t="n">
+        <v>0.03574757749122821</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J53" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>1494</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>0.004032258064516129</v>
+      </c>
+      <c r="I54" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J54" s="5" t="n">
+        <v>0.001451901191389071</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>0.03763440860215054</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J55" s="5" t="n">
+        <v>0.02825134476321248</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J56" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>1293</v>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>0.004662004662004662</v>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J57" s="5" t="n">
+        <v>0.002081647788877604</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="H58" s="5" t="n">
+        <v>0.006216006216006216</v>
+      </c>
+      <c r="I58" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J58" s="5" t="n">
+        <v>-0.003167057622931846</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
           <t>8624</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>いちよし証券</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n">
+      <c r="D59" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="H59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J59" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
         <v>46289</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E60" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="F60" s="4" t="n">
         <v>1686</v>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="G60" s="4" t="n">
         <v>1682</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H60" s="5" t="n">
         <v>-0.002372479240806643</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I60" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J60" s="5" t="n">
         <v>-0.004952836113933701</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>0.01423487544483986</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J61" s="5" t="n">
+        <v>0.004851811605901795</v>
       </c>
     </row>
   </sheetData>
@@ -3558,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3567,6 +4287,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3600,6 +4321,11 @@
           <t>2026-09-24</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -3624,6 +4350,9 @@
       <c r="F2" s="4" t="n">
         <v>2280</v>
       </c>
+      <c r="G2" s="4" t="n">
+        <v>2286</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3648,6 +4377,9 @@
       <c r="F3" s="4" t="n">
         <v>435</v>
       </c>
+      <c r="G3" s="4" t="n">
+        <v>436</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -3672,6 +4404,9 @@
       <c r="F4" s="4" t="n">
         <v>3135</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>2980</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -3696,6 +4431,9 @@
       <c r="F5" s="4" t="n">
         <v>2444</v>
       </c>
+      <c r="G5" s="4" t="n">
+        <v>2436</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -3720,6 +4458,9 @@
       <c r="F6" s="4" t="n">
         <v>1689</v>
       </c>
+      <c r="G6" s="4" t="n">
+        <v>1671</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -3744,6 +4485,9 @@
       <c r="F7" s="4" t="n">
         <v>4795</v>
       </c>
+      <c r="G7" s="4" t="n">
+        <v>4855</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -3768,6 +4512,9 @@
       <c r="F8" s="4" t="n">
         <v>2175</v>
       </c>
+      <c r="G8" s="4" t="n">
+        <v>2152</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -3792,6 +4539,9 @@
       <c r="F9" s="4" t="n">
         <v>2920</v>
       </c>
+      <c r="G9" s="4" t="n">
+        <v>2898</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -3816,6 +4566,9 @@
       <c r="F10" s="4" t="n">
         <v>2370.5</v>
       </c>
+      <c r="G10" s="4" t="n">
+        <v>2399</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -3840,6 +4593,9 @@
       <c r="F11" s="4" t="n">
         <v>6964</v>
       </c>
+      <c r="G11" s="4" t="n">
+        <v>6986</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3864,6 +4620,9 @@
       <c r="F12" s="4" t="n">
         <v>3825</v>
       </c>
+      <c r="G12" s="4" t="n">
+        <v>3871</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -3888,6 +4647,9 @@
       <c r="F13" s="4" t="n">
         <v>2466</v>
       </c>
+      <c r="G13" s="4" t="n">
+        <v>2527</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -3912,6 +4674,9 @@
       <c r="F14" s="4" t="n">
         <v>2060</v>
       </c>
+      <c r="G14" s="4" t="n">
+        <v>2067</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -3936,6 +4701,9 @@
       <c r="F15" s="4" t="n">
         <v>23605</v>
       </c>
+      <c r="G15" s="4" t="n">
+        <v>22975</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -3960,6 +4728,9 @@
       <c r="F16" s="4" t="n">
         <v>730</v>
       </c>
+      <c r="G16" s="4" t="n">
+        <v>675</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -3984,6 +4755,9 @@
       <c r="F17" s="4" t="n">
         <v>3375</v>
       </c>
+      <c r="G17" s="4" t="n">
+        <v>3325</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -4008,6 +4782,9 @@
       <c r="F18" s="4" t="n">
         <v>848</v>
       </c>
+      <c r="G18" s="4" t="n">
+        <v>880</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -4032,6 +4809,9 @@
       <c r="F19" s="4" t="n">
         <v>1494</v>
       </c>
+      <c r="G19" s="4" t="n">
+        <v>1544</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -4056,6 +4836,9 @@
       <c r="F20" s="4" t="n">
         <v>1293</v>
       </c>
+      <c r="G20" s="4" t="n">
+        <v>1295</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -4080,6 +4863,9 @@
       <c r="F21" s="4" t="n">
         <v>1682</v>
       </c>
+      <c r="G21" s="4" t="n">
+        <v>1710</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -4100,6 +4886,7 @@
       </c>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -4120,6 +4907,7 @@
       </c>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -4140,6 +4928,7 @@
       </c>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -4160,6 +4949,7 @@
       </c>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -4180,6 +4970,7 @@
       </c>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -4200,6 +4991,7 @@
       </c>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -4220,6 +5012,7 @@
       </c>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -4240,6 +5033,7 @@
       </c>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -4260,6 +5054,7 @@
       </c>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -4280,6 +5075,7 @@
       </c>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -4300,6 +5096,7 @@
       </c>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -4320,6 +5117,7 @@
       </c>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -4340,6 +5138,7 @@
       </c>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -4360,6 +5159,7 @@
       </c>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -4380,6 +5180,7 @@
       </c>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -4400,6 +5201,7 @@
       </c>
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -4420,6 +5222,7 @@
       </c>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -4440,6 +5243,7 @@
       </c>
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -4460,6 +5264,7 @@
       </c>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -4480,6 +5285,7 @@
       </c>
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record entry prices 2026-10-03
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2027,6 +2027,766 @@
       </c>
       <c r="J41" s="4" t="n">
         <v>430.2999877929688</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>証券、商品先物取引業</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>電気・ガス業</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>2345</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>1926</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>ライト工業</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>952</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="J47" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>3758</v>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>食料品</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>2119</v>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>輸送用機器</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="J50" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>1645.5</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>東京エレクトロン</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>12100</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>424</v>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>医薬品</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>90.7</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="J54" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>2791</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>2038</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="I57" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="J57" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="I59" s="4" t="n">
+        <v>4710</v>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="I60" s="4" t="n">
+        <v>3835</v>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>1165</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>430.2000122070313</v>
       </c>
     </row>
   </sheetData>
@@ -4278,7 +5038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5287,6 +6047,426 @@
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>1926</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>ライト工業</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>952</v>
+      </c>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>3835</v>
+      </c>
+      <c r="E43" s="4" t="n"/>
+      <c r="F43" s="4" t="n"/>
+      <c r="G43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>2119</v>
+      </c>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>424</v>
+      </c>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>2345</v>
+      </c>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="n">
+        <v>1645.5</v>
+      </c>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>4710</v>
+      </c>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n">
+        <v>2038</v>
+      </c>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>2791</v>
+      </c>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="E52" s="4" t="n"/>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="n">
+        <v>3758</v>
+      </c>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>東京エレクトロン</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="n">
+        <v>12100</v>
+      </c>
+      <c r="E59" s="4" t="n"/>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="n">
+        <v>1165</v>
+      </c>
+      <c r="E61" s="4" t="n"/>
+      <c r="F61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Performance check 2026-09-19 -> 2026-10-03
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -2800,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2981,34 +2981,34 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>システナ</t>
+          <t>丸大食品</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>440</v>
+        <v>2311</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>440</v>
+        <v>2119</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0</v>
+        <v>-0.08308091735179576</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.09222946186443712</v>
       </c>
     </row>
     <row r="6">
@@ -3026,25 +3026,25 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>440</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.01136363636363636</v>
+        <v>0</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>-0.01394399323676342</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="7">
@@ -3062,25 +3062,25 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>440</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.00909090909090909</v>
+        <v>-0.01136363636363636</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>-0.01847397292984715</v>
+        <v>-0.01394399323676342</v>
       </c>
     </row>
     <row r="8">
@@ -3089,34 +3089,34 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>3080</v>
+        <v>440</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>3080</v>
+        <v>436</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0</v>
+        <v>-0.00909090909090909</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.01847397292984715</v>
       </c>
     </row>
     <row r="9">
@@ -3125,34 +3125,34 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>46289</v>
+        <v>46298</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>3080</v>
+        <v>440</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>3135</v>
+        <v>424</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.01785714285714286</v>
+        <v>-0.03636363636363636</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.0152767859840158</v>
+        <v>-0.04551218087627772</v>
       </c>
     </row>
     <row r="10">
@@ -3170,25 +3170,25 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>3080</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>2980</v>
+        <v>3080</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.03246753246753246</v>
+        <v>0</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-0.04185059630647053</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="11">
@@ -3197,34 +3197,34 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>2426</v>
+        <v>3135</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>0.01785714285714286</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.0152767859840158</v>
       </c>
     </row>
     <row r="12">
@@ -3233,34 +3233,34 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>2444</v>
+        <v>2980</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.00741962077493817</v>
+        <v>-0.03246753246753246</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.004839263901811112</v>
+        <v>-0.04185059630647053</v>
       </c>
     </row>
     <row r="13">
@@ -3269,34 +3269,34 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>46291</v>
+        <v>46298</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>2426</v>
+        <v>3080</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>2436</v>
+        <v>3370</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.004122011541632316</v>
+        <v>0.09415584415584416</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>-0.005261052297305746</v>
+        <v>0.0850072996432028</v>
       </c>
     </row>
     <row r="14">
@@ -3305,12 +3305,12 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -3320,10 +3320,10 @@
         <v>2</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1700</v>
+        <v>2426</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>1700</v>
+        <v>2426</v>
       </c>
       <c r="H14" s="5" t="n">
         <v>0</v>
@@ -3341,12 +3341,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -3356,19 +3356,19 @@
         <v>5</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>1700</v>
+        <v>2426</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>1689</v>
+        <v>2444</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.006470588235294118</v>
+        <v>0.00741962077493817</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.009050945108421176</v>
+        <v>0.004839263901811112</v>
       </c>
     </row>
     <row r="16">
@@ -3377,12 +3377,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -3392,19 +3392,19 @@
         <v>7</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>1700</v>
+        <v>2426</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1671</v>
+        <v>2436</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.01705882352941177</v>
+        <v>0.004122011541632316</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>0.009383063838938062</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.02644188736834983</v>
+        <v>-0.005261052297305746</v>
       </c>
     </row>
     <row r="17">
@@ -3413,34 +3413,34 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>4775</v>
+        <v>2426</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>4775</v>
+        <v>2345</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0</v>
+        <v>-0.03338829348722176</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.04253683799986312</v>
       </c>
     </row>
     <row r="18">
@@ -3449,34 +3449,34 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>4775</v>
+        <v>1700</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>4795</v>
+        <v>1700</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.004188481675392671</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.001608124802265612</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="19">
@@ -3485,34 +3485,34 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4775</v>
+        <v>1700</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>4855</v>
+        <v>1689</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.01675392670157068</v>
+        <v>-0.006470588235294118</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.00737086286263262</v>
+        <v>-0.009050945108421176</v>
       </c>
     </row>
     <row r="20">
@@ -3521,34 +3521,34 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>2163</v>
+        <v>1700</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>2163</v>
+        <v>1671</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0</v>
+        <v>-0.01705882352941177</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.02644188736834983</v>
       </c>
     </row>
     <row r="21">
@@ -3557,34 +3557,34 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>46289</v>
+        <v>46298</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>2163</v>
+        <v>1700</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>2175</v>
+        <v>1645.5</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0.005547850208044383</v>
+        <v>-0.03205882352941176</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.002967493334917325</v>
+        <v>-0.04120736804205313</v>
       </c>
     </row>
     <row r="22">
@@ -3593,34 +3593,34 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2163</v>
+        <v>4775</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>2152</v>
+        <v>4775</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.005085529357374018</v>
+        <v>0</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.01446859319631208</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="23">
@@ -3629,34 +3629,34 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>2915</v>
+        <v>4775</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>2915</v>
+        <v>4795</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>0</v>
+        <v>0.004188481675392671</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.001608124802265612</v>
       </c>
     </row>
     <row r="24">
@@ -3665,34 +3665,34 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>2915</v>
+        <v>4775</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>2920</v>
+        <v>4855</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.001715265866209262</v>
+        <v>0.01675392670157068</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>-0.0008650910069177959</v>
+        <v>0.00737086286263262</v>
       </c>
     </row>
     <row r="25">
@@ -3701,34 +3701,34 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>46291</v>
+        <v>46298</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>2915</v>
+        <v>4775</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>2898</v>
+        <v>4710</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>-0.005831903945111492</v>
+        <v>-0.01361256544502618</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>-0.01521496778404955</v>
+        <v>-0.02276110995766754</v>
       </c>
     </row>
     <row r="26">
@@ -3737,12 +3737,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
@@ -3752,10 +3752,10 @@
         <v>2</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>2383.5</v>
+        <v>2163</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>2383.5</v>
+        <v>2163</v>
       </c>
       <c r="H26" s="5" t="n">
         <v>0</v>
@@ -3773,12 +3773,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
@@ -3788,19 +3788,19 @@
         <v>5</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>2383.5</v>
+        <v>2163</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>2370.5</v>
+        <v>2175</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>-0.005454164044472415</v>
+        <v>0.005547850208044383</v>
       </c>
       <c r="I27" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J27" s="5" t="n">
-        <v>-0.008034520917599472</v>
+        <v>0.002967493334917325</v>
       </c>
     </row>
     <row r="28">
@@ -3809,12 +3809,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
@@ -3824,19 +3824,19 @@
         <v>7</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>2383.5</v>
+        <v>2163</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>2399</v>
+        <v>2152</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.006503041745332494</v>
+        <v>-0.005085529357374018</v>
       </c>
       <c r="I28" s="5" t="n">
         <v>0.009383063838938062</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>-0.002880022093605568</v>
+        <v>-0.01446859319631208</v>
       </c>
     </row>
     <row r="29">
@@ -3845,34 +3845,34 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>6825</v>
+        <v>2163</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>6825</v>
+        <v>2038</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>0</v>
+        <v>-0.05779010633379565</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.06693865084643701</v>
       </c>
     </row>
     <row r="30">
@@ -3881,34 +3881,34 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>6825</v>
+        <v>2915</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>6964</v>
+        <v>2915</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.02036630036630037</v>
+        <v>0</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.01778594349317331</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="31">
@@ -3917,34 +3917,34 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>6825</v>
+        <v>2915</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>6986</v>
+        <v>2920</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>0.02358974358974359</v>
+        <v>0.001715265866209262</v>
       </c>
       <c r="I31" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.01420667975080553</v>
+        <v>-0.0008650910069177959</v>
       </c>
     </row>
     <row r="32">
@@ -3953,34 +3953,34 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>5105</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>ＴＯＹＯ　ＴＩＲＥ</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>3804</v>
+        <v>2915</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>3804</v>
+        <v>2898</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0</v>
+        <v>-0.005831903945111492</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.01521496778404955</v>
       </c>
     </row>
     <row r="33">
@@ -3989,34 +3989,34 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>5105</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>ＴＯＹＯ　ＴＩＲＥ</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>46289</v>
+        <v>46298</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3804</v>
+        <v>2915</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>3825</v>
+        <v>2791</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>0.005520504731861199</v>
+        <v>-0.04253859348198971</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>0.002940147858734141</v>
+        <v>-0.05168713799463107</v>
       </c>
     </row>
     <row r="34">
@@ -4025,34 +4025,34 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>5105</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ＴＯＹＯ　ＴＩＲＥ</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>3804</v>
+        <v>2383.5</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>3871</v>
+        <v>2383.5</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.0176130389064143</v>
+        <v>0</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>0.00822997506747624</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="35">
@@ -4061,34 +4061,34 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>2454</v>
+        <v>2383.5</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>2454</v>
+        <v>2370.5</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>0</v>
+        <v>-0.005454164044472415</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.008034520917599472</v>
       </c>
     </row>
     <row r="36">
@@ -4097,34 +4097,34 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2454</v>
+        <v>2383.5</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>2466</v>
+        <v>2399</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.004889975550122249</v>
+        <v>0.006503041745332494</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.002309618676995191</v>
+        <v>-0.002880022093605568</v>
       </c>
     </row>
     <row r="37">
@@ -4133,34 +4133,34 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>46291</v>
+        <v>46298</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>2454</v>
+        <v>2383.5</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2527</v>
+        <v>2245</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>0.02974735126324368</v>
+        <v>-0.05810782462764841</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.02036428742430562</v>
+        <v>-0.06725636914028978</v>
       </c>
     </row>
     <row r="38">
@@ -4169,12 +4169,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
@@ -4184,10 +4184,10 @@
         <v>2</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>2060</v>
+        <v>6825</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>2060</v>
+        <v>6825</v>
       </c>
       <c r="H38" s="5" t="n">
         <v>0</v>
@@ -4205,12 +4205,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
@@ -4220,19 +4220,19 @@
         <v>5</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2060</v>
+        <v>6825</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>2060</v>
+        <v>6964</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>0</v>
+        <v>0.02036630036630037</v>
       </c>
       <c r="I39" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J39" s="5" t="n">
-        <v>-0.002580356873127058</v>
+        <v>0.01778594349317331</v>
       </c>
     </row>
     <row r="40">
@@ -4241,12 +4241,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
@@ -4256,19 +4256,19 @@
         <v>7</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2060</v>
+        <v>6825</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>2067</v>
+        <v>6986</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.003398058252427184</v>
+        <v>0.02358974358974359</v>
       </c>
       <c r="I40" s="5" t="n">
         <v>0.009383063838938062</v>
       </c>
       <c r="J40" s="5" t="n">
-        <v>-0.005985005586510878</v>
+        <v>0.01420667975080553</v>
       </c>
     </row>
     <row r="41">
@@ -4277,34 +4277,34 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>22795</v>
+        <v>6825</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>22795</v>
+        <v>7061</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>0</v>
+        <v>0.03457875457875458</v>
       </c>
       <c r="I41" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J41" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.02543021006611322</v>
       </c>
     </row>
     <row r="42">
@@ -4313,34 +4313,34 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>22795</v>
+        <v>3804</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>23605</v>
+        <v>3804</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.03553410835709585</v>
+        <v>0</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.0329537514839688</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="43">
@@ -4349,34 +4349,34 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>22795</v>
+        <v>3804</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>22975</v>
+        <v>3825</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>0.007896468523799079</v>
+        <v>0.005520504731861199</v>
       </c>
       <c r="I43" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J43" s="5" t="n">
-        <v>-0.001486595315138983</v>
+        <v>0.002940147858734141</v>
       </c>
     </row>
     <row r="44">
@@ -4385,34 +4385,34 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>723</v>
+        <v>3804</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>723</v>
+        <v>3871</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0</v>
+        <v>0.0176130389064143</v>
       </c>
       <c r="I44" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J44" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.00822997506747624</v>
       </c>
     </row>
     <row r="45">
@@ -4421,34 +4421,34 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>5105</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>ＴＯＹＯ　ＴＩＲＥ</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>46289</v>
+        <v>46298</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>723</v>
+        <v>3804</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>730</v>
+        <v>3905</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>0.009681881051175657</v>
+        <v>0.02655099894847529</v>
       </c>
       <c r="I45" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J45" s="5" t="n">
-        <v>0.007101524178048599</v>
+        <v>0.01740245443583393</v>
       </c>
     </row>
     <row r="46">
@@ -4457,34 +4457,34 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>723</v>
+        <v>2454</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>675</v>
+        <v>2454</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>-0.06639004149377593</v>
+        <v>0</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>-0.075773105332714</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="47">
@@ -4493,34 +4493,34 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>3370</v>
+        <v>2454</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>3370</v>
+        <v>2466</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>0</v>
+        <v>0.004889975550122249</v>
       </c>
       <c r="I47" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.002309618676995191</v>
       </c>
     </row>
     <row r="48">
@@ -4529,34 +4529,34 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>3370</v>
+        <v>2454</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>3375</v>
+        <v>2527</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.001483679525222552</v>
+        <v>0.02974735126324368</v>
       </c>
       <c r="I48" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>-0.001096677347904506</v>
+        <v>0.02036428742430562</v>
       </c>
     </row>
     <row r="49">
@@ -4565,34 +4565,34 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>5195</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>バンドー化学</t>
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>46291</v>
+        <v>46298</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>3370</v>
+        <v>2454</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>3325</v>
+        <v>2450</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>-0.01335311572700297</v>
+        <v>-0.00162999185004075</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>-0.02273617956594103</v>
+        <v>-0.01077853636268211</v>
       </c>
     </row>
     <row r="50">
@@ -4601,12 +4601,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D50" s="2" t="n">
@@ -4616,10 +4616,10 @@
         <v>2</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>842</v>
+        <v>2060</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>842</v>
+        <v>2060</v>
       </c>
       <c r="H50" s="5" t="n">
         <v>0</v>
@@ -4637,12 +4637,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D51" s="2" t="n">
@@ -4652,19 +4652,19 @@
         <v>5</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>842</v>
+        <v>2060</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>848</v>
+        <v>2060</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>0.007125890736342043</v>
+        <v>0</v>
       </c>
       <c r="I51" s="5" t="n">
         <v>0.002580356873127058</v>
       </c>
       <c r="J51" s="5" t="n">
-        <v>0.004545533863214985</v>
+        <v>-0.002580356873127058</v>
       </c>
     </row>
     <row r="52">
@@ -4673,12 +4673,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D52" s="2" t="n">
@@ -4688,19 +4688,19 @@
         <v>7</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>842</v>
+        <v>2060</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>880</v>
+        <v>2067</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>0.04513064133016627</v>
+        <v>0.003398058252427184</v>
       </c>
       <c r="I52" s="5" t="n">
         <v>0.009383063838938062</v>
       </c>
       <c r="J52" s="5" t="n">
-        <v>0.03574757749122821</v>
+        <v>-0.005985005586510878</v>
       </c>
     </row>
     <row r="53">
@@ -4709,34 +4709,34 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>5445</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>東京鐵鋼</t>
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>46286</v>
+        <v>46298</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>1488</v>
+        <v>2060</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>1488</v>
+        <v>1950</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>0</v>
+        <v>-0.05339805825242718</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.06254660276506854</v>
       </c>
     </row>
     <row r="54">
@@ -4745,34 +4745,34 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>5706</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>三井金属</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>46289</v>
+        <v>46286</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>1488</v>
+        <v>22795</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>1494</v>
+        <v>22795</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>0.004032258064516129</v>
+        <v>0</v>
       </c>
       <c r="I54" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J54" s="5" t="n">
-        <v>0.001451901191389071</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="55">
@@ -4781,34 +4781,34 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>5706</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>三井金属</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>46291</v>
+        <v>46289</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>1488</v>
+        <v>22795</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>1544</v>
+        <v>23605</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>0.03763440860215054</v>
+        <v>0.03553410835709585</v>
       </c>
       <c r="I55" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J55" s="5" t="n">
-        <v>0.02825134476321248</v>
+        <v>0.0329537514839688</v>
       </c>
     </row>
     <row r="56">
@@ -4817,34 +4817,34 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>5706</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>三井金属</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>46286</v>
+        <v>46291</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>1287</v>
+        <v>22795</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>1287</v>
+        <v>22975</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>0</v>
+        <v>0.007896468523799079</v>
       </c>
       <c r="I56" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J56" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>-0.001486595315138983</v>
       </c>
     </row>
     <row r="57">
@@ -4853,34 +4853,34 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>5706</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>三井金属</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>46289</v>
+        <v>46298</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>1287</v>
+        <v>22795</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>1293</v>
+        <v>2553.5</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>0.004662004662004662</v>
+        <v>-0.8879798201359947</v>
       </c>
       <c r="I57" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.00914854451264136</v>
       </c>
       <c r="J57" s="5" t="n">
-        <v>0.002081647788877604</v>
+        <v>-0.8971283646486361</v>
       </c>
     </row>
     <row r="58">
@@ -4889,34 +4889,34 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>6200</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>インソース</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>46291</v>
+        <v>46286</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>1287</v>
+        <v>723</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>1295</v>
+        <v>723</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>0.006216006216006216</v>
+        <v>0</v>
       </c>
       <c r="I58" s="5" t="n">
-        <v>0.009383063838938062</v>
+        <v>-1.333413569986163e-16</v>
       </c>
       <c r="J58" s="5" t="n">
-        <v>-0.003167057622931846</v>
+        <v>1.333413569986163e-16</v>
       </c>
     </row>
     <row r="59">
@@ -4925,34 +4925,34 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>8624</t>
+          <t>6200</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>いちよし証券</t>
+          <t>インソース</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>1686</v>
+        <v>723</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>1686</v>
+        <v>730</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>0</v>
+        <v>0.009681881051175657</v>
       </c>
       <c r="I59" s="5" t="n">
-        <v>-1.333413569986163e-16</v>
+        <v>0.002580356873127058</v>
       </c>
       <c r="J59" s="5" t="n">
-        <v>1.333413569986163e-16</v>
+        <v>0.007101524178048599</v>
       </c>
     </row>
     <row r="60">
@@ -4961,34 +4961,34 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>8624</t>
+          <t>6200</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>いちよし証券</t>
+          <t>インソース</t>
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>1686</v>
+        <v>723</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>1682</v>
+        <v>675</v>
       </c>
       <c r="H60" s="5" t="n">
-        <v>-0.002372479240806643</v>
+        <v>-0.06639004149377593</v>
       </c>
       <c r="I60" s="5" t="n">
-        <v>0.002580356873127058</v>
+        <v>0.009383063838938062</v>
       </c>
       <c r="J60" s="5" t="n">
-        <v>-0.004952836113933701</v>
+        <v>-0.075773105332714</v>
       </c>
     </row>
     <row r="61">
@@ -4997,34 +4997,754 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>723</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>-0.07330567081604426</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J61" s="5" t="n">
+        <v>-0.08245421532868562</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="H62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J62" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>3375</v>
+      </c>
+      <c r="H63" s="5" t="n">
+        <v>0.001483679525222552</v>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>-0.001096677347904506</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>-0.01335311572700297</v>
+      </c>
+      <c r="I64" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J64" s="5" t="n">
+        <v>-0.02273617956594103</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>-0.09495548961424333</v>
+      </c>
+      <c r="I65" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J65" s="5" t="n">
+        <v>-0.1041040341268847</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="H66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J66" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>848</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>0.007125890736342043</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>0.004545533863214985</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="H68" s="5" t="n">
+        <v>0.04513064133016627</v>
+      </c>
+      <c r="I68" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J68" s="5" t="n">
+        <v>0.03574757749122821</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>842</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>863</v>
+      </c>
+      <c r="H69" s="5" t="n">
+        <v>0.02494061757719715</v>
+      </c>
+      <c r="I69" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J69" s="5" t="n">
+        <v>0.01579207306455579</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="H70" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J70" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>1494</v>
+      </c>
+      <c r="H71" s="5" t="n">
+        <v>0.004032258064516129</v>
+      </c>
+      <c r="I71" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J71" s="5" t="n">
+        <v>0.001451901191389071</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="H72" s="5" t="n">
+        <v>0.03763440860215054</v>
+      </c>
+      <c r="I72" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J72" s="5" t="n">
+        <v>0.02825134476321248</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>1488</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="H73" s="5" t="n">
+        <v>-0.01478494623655914</v>
+      </c>
+      <c r="I73" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J73" s="5" t="n">
+        <v>-0.0239334907492005</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="H74" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J74" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>1293</v>
+      </c>
+      <c r="H75" s="5" t="n">
+        <v>0.004662004662004662</v>
+      </c>
+      <c r="I75" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J75" s="5" t="n">
+        <v>0.002081647788877604</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="H76" s="5" t="n">
+        <v>0.006216006216006216</v>
+      </c>
+      <c r="I76" s="5" t="n">
+        <v>0.009383063838938062</v>
+      </c>
+      <c r="J76" s="5" t="n">
+        <v>-0.003167057622931846</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F77" s="4" t="n">
+        <v>1287</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="H77" s="5" t="n">
+        <v>-0.06060606060606061</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J77" s="5" t="n">
+        <v>-0.06975460511870196</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
           <t>8624</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>いちよし証券</t>
         </is>
       </c>
-      <c r="D61" s="2" t="n">
+      <c r="D78" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="H78" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="5" t="n">
+        <v>-1.333413569986163e-16</v>
+      </c>
+      <c r="J78" s="5" t="n">
+        <v>1.333413569986163e-16</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>1682</v>
+      </c>
+      <c r="H79" s="5" t="n">
+        <v>-0.002372479240806643</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>0.002580356873127058</v>
+      </c>
+      <c r="J79" s="5" t="n">
+        <v>-0.004952836113933701</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
         <v>46291</v>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="E80" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F61" s="4" t="n">
+      <c r="F80" s="4" t="n">
         <v>1686</v>
       </c>
-      <c r="G61" s="4" t="n">
+      <c r="G80" s="4" t="n">
         <v>1710</v>
       </c>
-      <c r="H61" s="5" t="n">
+      <c r="H80" s="5" t="n">
         <v>0.01423487544483986</v>
       </c>
-      <c r="I61" s="5" t="n">
+      <c r="I80" s="5" t="n">
         <v>0.009383063838938062</v>
       </c>
-      <c r="J61" s="5" t="n">
+      <c r="J80" s="5" t="n">
         <v>0.004851811605901795</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>1686</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <v>-0.05041518386714116</v>
+      </c>
+      <c r="I81" s="5" t="n">
+        <v>0.00914854451264136</v>
+      </c>
+      <c r="J81" s="5" t="n">
+        <v>-0.05956372837978252</v>
       </c>
     </row>
   </sheetData>
@@ -5038,7 +5758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5048,6 +5768,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5086,6 +5807,11 @@
           <t>2026-09-26</t>
         </is>
       </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -5113,6 +5839,9 @@
       <c r="G2" s="4" t="n">
         <v>2286</v>
       </c>
+      <c r="H2" s="4" t="n">
+        <v>2119</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -5140,6 +5869,9 @@
       <c r="G3" s="4" t="n">
         <v>436</v>
       </c>
+      <c r="H3" s="4" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -5167,6 +5899,9 @@
       <c r="G4" s="4" t="n">
         <v>2980</v>
       </c>
+      <c r="H4" s="4" t="n">
+        <v>3370</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -5194,6 +5929,9 @@
       <c r="G5" s="4" t="n">
         <v>2436</v>
       </c>
+      <c r="H5" s="4" t="n">
+        <v>2345</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -5221,6 +5959,9 @@
       <c r="G6" s="4" t="n">
         <v>1671</v>
       </c>
+      <c r="H6" s="4" t="n">
+        <v>1645.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -5248,6 +5989,9 @@
       <c r="G7" s="4" t="n">
         <v>4855</v>
       </c>
+      <c r="H7" s="4" t="n">
+        <v>4710</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -5275,6 +6019,9 @@
       <c r="G8" s="4" t="n">
         <v>2152</v>
       </c>
+      <c r="H8" s="4" t="n">
+        <v>2038</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -5302,6 +6049,9 @@
       <c r="G9" s="4" t="n">
         <v>2898</v>
       </c>
+      <c r="H9" s="4" t="n">
+        <v>2791</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -5329,6 +6079,9 @@
       <c r="G10" s="4" t="n">
         <v>2399</v>
       </c>
+      <c r="H10" s="4" t="n">
+        <v>2245</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -5356,6 +6109,9 @@
       <c r="G11" s="4" t="n">
         <v>6986</v>
       </c>
+      <c r="H11" s="4" t="n">
+        <v>7061</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -5383,6 +6139,9 @@
       <c r="G12" s="4" t="n">
         <v>3871</v>
       </c>
+      <c r="H12" s="4" t="n">
+        <v>3905</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -5410,6 +6169,9 @@
       <c r="G13" s="4" t="n">
         <v>2527</v>
       </c>
+      <c r="H13" s="4" t="n">
+        <v>2450</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -5437,6 +6199,9 @@
       <c r="G14" s="4" t="n">
         <v>2067</v>
       </c>
+      <c r="H14" s="4" t="n">
+        <v>1950</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -5464,6 +6229,9 @@
       <c r="G15" s="4" t="n">
         <v>22975</v>
       </c>
+      <c r="H15" s="4" t="n">
+        <v>2553.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -5491,6 +6259,9 @@
       <c r="G16" s="4" t="n">
         <v>675</v>
       </c>
+      <c r="H16" s="4" t="n">
+        <v>670</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -5518,6 +6289,9 @@
       <c r="G17" s="4" t="n">
         <v>3325</v>
       </c>
+      <c r="H17" s="4" t="n">
+        <v>3050</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -5545,6 +6319,9 @@
       <c r="G18" s="4" t="n">
         <v>880</v>
       </c>
+      <c r="H18" s="4" t="n">
+        <v>863</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -5572,6 +6349,9 @@
       <c r="G19" s="4" t="n">
         <v>1544</v>
       </c>
+      <c r="H19" s="4" t="n">
+        <v>1466</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -5599,6 +6379,9 @@
       <c r="G20" s="4" t="n">
         <v>1295</v>
       </c>
+      <c r="H20" s="4" t="n">
+        <v>1209</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -5625,6 +6408,9 @@
       </c>
       <c r="G21" s="4" t="n">
         <v>1710</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>1601</v>
       </c>
     </row>
     <row r="22">
@@ -5647,6 +6433,7 @@
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -5668,6 +6455,7 @@
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -5689,6 +6477,7 @@
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -5710,6 +6499,7 @@
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -5731,6 +6521,7 @@
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -5752,6 +6543,7 @@
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -5773,6 +6565,7 @@
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -5794,6 +6587,7 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -5815,6 +6609,7 @@
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -5836,6 +6631,7 @@
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -5857,6 +6653,7 @@
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -5878,6 +6675,7 @@
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -5899,6 +6697,7 @@
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -5920,6 +6719,7 @@
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -5941,6 +6741,7 @@
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -5962,6 +6763,7 @@
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -5983,6 +6785,7 @@
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -6004,6 +6807,7 @@
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -6025,6 +6829,7 @@
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -6046,6 +6851,7 @@
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
+      <c r="H41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -6067,6 +6873,7 @@
       <c r="E42" s="4" t="n"/>
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -6088,6 +6895,7 @@
       <c r="E43" s="4" t="n"/>
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
+      <c r="H43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -6109,6 +6917,7 @@
       <c r="E44" s="4" t="n"/>
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -6130,6 +6939,7 @@
       <c r="E45" s="4" t="n"/>
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -6151,6 +6961,7 @@
       <c r="E46" s="4" t="n"/>
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -6172,6 +6983,7 @@
       <c r="E47" s="4" t="n"/>
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -6193,6 +7005,7 @@
       <c r="E48" s="4" t="n"/>
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -6214,6 +7027,7 @@
       <c r="E49" s="4" t="n"/>
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -6235,6 +7049,7 @@
       <c r="E50" s="4" t="n"/>
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -6256,6 +7071,7 @@
       <c r="E51" s="4" t="n"/>
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -6277,6 +7093,7 @@
       <c r="E52" s="4" t="n"/>
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -6298,6 +7115,7 @@
       <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -6319,6 +7137,7 @@
       <c r="E54" s="4" t="n"/>
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -6340,6 +7159,7 @@
       <c r="E55" s="4" t="n"/>
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -6361,6 +7181,7 @@
       <c r="E56" s="4" t="n"/>
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -6382,6 +7203,7 @@
       <c r="E57" s="4" t="n"/>
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -6403,6 +7225,7 @@
       <c r="E58" s="4" t="n"/>
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -6424,6 +7247,7 @@
       <c r="E59" s="4" t="n"/>
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -6445,6 +7269,7 @@
       <c r="E60" s="4" t="n"/>
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -6466,6 +7291,7 @@
       <c r="E61" s="4" t="n"/>
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Performance check 2026-09-26 -> 2026-10-03
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -2800,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5745,6 +5745,726 @@
       </c>
       <c r="J81" s="5" t="n">
         <v>-0.05956372837978252</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F82" s="4" t="n">
+        <v>2286</v>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>2119</v>
+      </c>
+      <c r="H82" s="5" t="n">
+        <v>-0.07305336832895888</v>
+      </c>
+      <c r="I82" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J82" s="5" t="n">
+        <v>-0.07282102905688422</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>436</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>424</v>
+      </c>
+      <c r="H83" s="5" t="n">
+        <v>-0.02752293577981652</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J83" s="5" t="n">
+        <v>-0.02729059650774185</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F84" s="4" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="H84" s="5" t="n">
+        <v>0.1308724832214765</v>
+      </c>
+      <c r="I84" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J84" s="5" t="n">
+        <v>0.1311048224935512</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F85" s="4" t="n">
+        <v>2436</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>2345</v>
+      </c>
+      <c r="H85" s="5" t="n">
+        <v>-0.03735632183908046</v>
+      </c>
+      <c r="I85" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J85" s="5" t="n">
+        <v>-0.0371239825670058</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>1645.5</v>
+      </c>
+      <c r="H86" s="5" t="n">
+        <v>-0.01526032315978456</v>
+      </c>
+      <c r="I86" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J86" s="5" t="n">
+        <v>-0.01502798388770989</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F87" s="4" t="n">
+        <v>4855</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>4710</v>
+      </c>
+      <c r="H87" s="5" t="n">
+        <v>-0.02986611740473738</v>
+      </c>
+      <c r="I87" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J87" s="5" t="n">
+        <v>-0.02963377813266272</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F88" s="4" t="n">
+        <v>2152</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>2038</v>
+      </c>
+      <c r="H88" s="5" t="n">
+        <v>-0.05297397769516728</v>
+      </c>
+      <c r="I88" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J88" s="5" t="n">
+        <v>-0.05274163842309262</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F89" s="4" t="n">
+        <v>2898</v>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>2791</v>
+      </c>
+      <c r="H89" s="5" t="n">
+        <v>-0.03692201518288475</v>
+      </c>
+      <c r="I89" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J89" s="5" t="n">
+        <v>-0.03668967591081009</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F90" s="4" t="n">
+        <v>2399</v>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="H90" s="5" t="n">
+        <v>-0.06419341392246769</v>
+      </c>
+      <c r="I90" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J90" s="5" t="n">
+        <v>-0.06396107465039302</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>5101</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>横浜ゴム</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F91" s="4" t="n">
+        <v>6986</v>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>7061</v>
+      </c>
+      <c r="H91" s="5" t="n">
+        <v>0.0107357572287432</v>
+      </c>
+      <c r="I91" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J91" s="5" t="n">
+        <v>0.01096809650081787</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="H92" s="5" t="n">
+        <v>-0.03047091412742382</v>
+      </c>
+      <c r="I92" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J92" s="5" t="n">
+        <v>-0.03023857485534916</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>5445</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>東京鐵鋼</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F93" s="4" t="n">
+        <v>2067</v>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>1950</v>
+      </c>
+      <c r="H93" s="5" t="n">
+        <v>-0.05660377358490566</v>
+      </c>
+      <c r="I93" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J93" s="5" t="n">
+        <v>-0.056371434312831</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F94" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="G94" s="4" t="n">
+        <v>2553.5</v>
+      </c>
+      <c r="H94" s="5" t="n">
+        <v>-0.8888574537540805</v>
+      </c>
+      <c r="I94" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J94" s="5" t="n">
+        <v>-0.8886251144820059</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F95" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="G95" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="H95" s="5" t="n">
+        <v>-0.007407407407407408</v>
+      </c>
+      <c r="I95" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J95" s="5" t="n">
+        <v>-0.00717506813533274</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="G96" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="H96" s="5" t="n">
+        <v>-0.08270676691729323</v>
+      </c>
+      <c r="I96" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J96" s="5" t="n">
+        <v>-0.08247442764521856</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F97" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="G97" s="4" t="n">
+        <v>863</v>
+      </c>
+      <c r="H97" s="5" t="n">
+        <v>-0.01931818181818182</v>
+      </c>
+      <c r="I97" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J97" s="5" t="n">
+        <v>-0.01908584254610715</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F98" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="G98" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="H98" s="5" t="n">
+        <v>-0.05051813471502591</v>
+      </c>
+      <c r="I98" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J98" s="5" t="n">
+        <v>-0.05028579544295124</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E99" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F99" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="G99" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="H99" s="5" t="n">
+        <v>-0.06640926640926641</v>
+      </c>
+      <c r="I99" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J99" s="5" t="n">
+        <v>-0.06617692713719174</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F100" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G100" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="H100" s="5" t="n">
+        <v>-0.06374269005847953</v>
+      </c>
+      <c r="I100" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J100" s="5" t="n">
+        <v>-0.06351035078640486</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F101" s="4" t="n">
+        <v>1191</v>
+      </c>
+      <c r="G101" s="4" t="n">
+        <v>1165</v>
+      </c>
+      <c r="H101" s="5" t="n">
+        <v>-0.0218303946263644</v>
+      </c>
+      <c r="I101" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J101" s="5" t="n">
+        <v>-0.02159805535428973</v>
       </c>
     </row>
   </sheetData>
@@ -6433,7 +7153,9 @@
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
+      <c r="H22" s="4" t="n">
+        <v>2119</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -6455,7 +7177,9 @@
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
+      <c r="H23" s="4" t="n">
+        <v>424</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -6477,7 +7201,9 @@
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
+      <c r="H24" s="4" t="n">
+        <v>3370</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -6499,7 +7225,9 @@
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
+      <c r="H25" s="4" t="n">
+        <v>2345</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -6521,7 +7249,9 @@
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
+      <c r="H26" s="4" t="n">
+        <v>1645.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -6543,7 +7273,9 @@
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
+      <c r="H27" s="4" t="n">
+        <v>4710</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -6565,7 +7297,9 @@
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
+      <c r="H28" s="4" t="n">
+        <v>2038</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -6587,7 +7321,9 @@
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
+      <c r="H29" s="4" t="n">
+        <v>2791</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -6609,7 +7345,9 @@
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
+      <c r="H30" s="4" t="n">
+        <v>2245</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -6631,7 +7369,9 @@
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
+      <c r="H31" s="4" t="n">
+        <v>7061</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -6653,7 +7393,9 @@
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
+      <c r="H32" s="4" t="n">
+        <v>2450</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -6675,7 +7417,9 @@
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
+      <c r="H33" s="4" t="n">
+        <v>1950</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -6697,7 +7441,9 @@
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
+      <c r="H34" s="4" t="n">
+        <v>2553.5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -6719,7 +7465,9 @@
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="n"/>
+      <c r="H35" s="4" t="n">
+        <v>670</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -6741,7 +7489,9 @@
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
+      <c r="H36" s="4" t="n">
+        <v>3050</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -6763,7 +7513,9 @@
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
+      <c r="H37" s="4" t="n">
+        <v>863</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -6785,7 +7537,9 @@
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
+      <c r="H38" s="4" t="n">
+        <v>1466</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -6807,7 +7561,9 @@
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
+      <c r="H39" s="4" t="n">
+        <v>1209</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -6829,7 +7585,9 @@
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
+      <c r="H40" s="4" t="n">
+        <v>1601</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -6851,7 +7609,9 @@
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="n"/>
       <c r="G41" s="4" t="n"/>
-      <c r="H41" s="4" t="n"/>
+      <c r="H41" s="4" t="n">
+        <v>1165</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">

</xml_diff>

<commit_message>
Performance check 2026-09-26 -> 2026-10-05
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -2800,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6509,34 +6509,34 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>システナ</t>
+          <t>丸大食品</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>436</v>
+        <v>2286</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>424</v>
+        <v>2125</v>
       </c>
       <c r="H103" s="5" t="n">
-        <v>-0.02752293577981652</v>
+        <v>-0.07042869641294838</v>
       </c>
       <c r="I103" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J103" s="5" t="n">
-        <v>-0.02729059650774185</v>
+        <v>-0.08437245697583907</v>
       </c>
     </row>
     <row r="104">
@@ -6545,12 +6545,12 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
@@ -6560,19 +6560,19 @@
         <v>7</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>2980</v>
+        <v>436</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>3370</v>
+        <v>424</v>
       </c>
       <c r="H104" s="5" t="n">
-        <v>0.1308724832214765</v>
+        <v>-0.02752293577981652</v>
       </c>
       <c r="I104" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J104" s="5" t="n">
-        <v>0.1311048224935512</v>
+        <v>-0.02729059650774185</v>
       </c>
     </row>
     <row r="105">
@@ -6581,34 +6581,34 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>2436</v>
+        <v>436</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>2345</v>
+        <v>422</v>
       </c>
       <c r="H105" s="5" t="n">
-        <v>-0.03735632183908046</v>
+        <v>-0.03211009174311927</v>
       </c>
       <c r="I105" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J105" s="5" t="n">
-        <v>-0.0371239825670058</v>
+        <v>-0.04605385230600996</v>
       </c>
     </row>
     <row r="106">
@@ -6617,12 +6617,12 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D106" s="2" t="n">
@@ -6632,19 +6632,19 @@
         <v>7</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>1671</v>
+        <v>2980</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>1645.5</v>
+        <v>3370</v>
       </c>
       <c r="H106" s="5" t="n">
-        <v>-0.01526032315978456</v>
+        <v>0.1308724832214765</v>
       </c>
       <c r="I106" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J106" s="5" t="n">
-        <v>-0.01502798388770989</v>
+        <v>0.1311048224935512</v>
       </c>
     </row>
     <row r="107">
@@ -6653,34 +6653,34 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>4855</v>
+        <v>2980</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>4710</v>
+        <v>3360</v>
       </c>
       <c r="H107" s="5" t="n">
-        <v>-0.02986611740473738</v>
+        <v>0.1275167785234899</v>
       </c>
       <c r="I107" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J107" s="5" t="n">
-        <v>-0.02963377813266272</v>
+        <v>0.1135730179605993</v>
       </c>
     </row>
     <row r="108">
@@ -6689,12 +6689,12 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D108" s="2" t="n">
@@ -6704,19 +6704,19 @@
         <v>7</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>2152</v>
+        <v>2436</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>2038</v>
+        <v>2345</v>
       </c>
       <c r="H108" s="5" t="n">
-        <v>-0.05297397769516728</v>
+        <v>-0.03735632183908046</v>
       </c>
       <c r="I108" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J108" s="5" t="n">
-        <v>-0.05274163842309262</v>
+        <v>-0.0371239825670058</v>
       </c>
     </row>
     <row r="109">
@@ -6725,34 +6725,34 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>2898</v>
+        <v>2436</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>2791</v>
+        <v>2362</v>
       </c>
       <c r="H109" s="5" t="n">
-        <v>-0.03692201518288475</v>
+        <v>-0.03037766830870279</v>
       </c>
       <c r="I109" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J109" s="5" t="n">
-        <v>-0.03668967591081009</v>
+        <v>-0.04432142887159348</v>
       </c>
     </row>
     <row r="110">
@@ -6761,12 +6761,12 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D110" s="2" t="n">
@@ -6776,19 +6776,19 @@
         <v>7</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>2399</v>
+        <v>1671</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>2245</v>
+        <v>1645.5</v>
       </c>
       <c r="H110" s="5" t="n">
-        <v>-0.06419341392246769</v>
+        <v>-0.01526032315978456</v>
       </c>
       <c r="I110" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J110" s="5" t="n">
-        <v>-0.06396107465039302</v>
+        <v>-0.01502798388770989</v>
       </c>
     </row>
     <row r="111">
@@ -6797,34 +6797,34 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>5101</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>横浜ゴム</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>6986</v>
+        <v>1671</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>7061</v>
+        <v>1620.5</v>
       </c>
       <c r="H111" s="5" t="n">
-        <v>0.0107357572287432</v>
+        <v>-0.03022142429682825</v>
       </c>
       <c r="I111" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J111" s="5" t="n">
-        <v>0.01096809650081787</v>
+        <v>-0.04416518485971893</v>
       </c>
     </row>
     <row r="112">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D112" s="2" t="n">
@@ -6848,19 +6848,19 @@
         <v>7</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>2527</v>
+        <v>4855</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>2450</v>
+        <v>4710</v>
       </c>
       <c r="H112" s="5" t="n">
-        <v>-0.03047091412742382</v>
+        <v>-0.02986611740473738</v>
       </c>
       <c r="I112" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J112" s="5" t="n">
-        <v>-0.03023857485534916</v>
+        <v>-0.02963377813266272</v>
       </c>
     </row>
     <row r="113">
@@ -6869,34 +6869,34 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>5445</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>東京鐵鋼</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F113" s="4" t="n">
-        <v>2067</v>
+        <v>4855</v>
       </c>
       <c r="G113" s="4" t="n">
-        <v>1950</v>
+        <v>4655</v>
       </c>
       <c r="H113" s="5" t="n">
-        <v>-0.05660377358490566</v>
+        <v>-0.0411946446961895</v>
       </c>
       <c r="I113" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J113" s="5" t="n">
-        <v>-0.056371434312831</v>
+        <v>-0.05513840525908019</v>
       </c>
     </row>
     <row r="114">
@@ -6905,12 +6905,12 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>5706</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>三井金属</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D114" s="2" t="n">
@@ -6920,19 +6920,19 @@
         <v>7</v>
       </c>
       <c r="F114" s="4" t="n">
-        <v>22975</v>
+        <v>2152</v>
       </c>
       <c r="G114" s="4" t="n">
-        <v>2553.5</v>
+        <v>2038</v>
       </c>
       <c r="H114" s="5" t="n">
-        <v>-0.8888574537540805</v>
+        <v>-0.05297397769516728</v>
       </c>
       <c r="I114" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J114" s="5" t="n">
-        <v>-0.8886251144820059</v>
+        <v>-0.05274163842309262</v>
       </c>
     </row>
     <row r="115">
@@ -6941,34 +6941,34 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F115" s="4" t="n">
-        <v>675</v>
+        <v>2152</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>670</v>
+        <v>2022</v>
       </c>
       <c r="H115" s="5" t="n">
-        <v>-0.007407407407407408</v>
+        <v>-0.0604089219330855</v>
       </c>
       <c r="I115" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J115" s="5" t="n">
-        <v>-0.00717506813533274</v>
+        <v>-0.07435268249597619</v>
       </c>
     </row>
     <row r="116">
@@ -6977,12 +6977,12 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D116" s="2" t="n">
@@ -6992,19 +6992,19 @@
         <v>7</v>
       </c>
       <c r="F116" s="4" t="n">
-        <v>3325</v>
+        <v>2898</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>3050</v>
+        <v>2791</v>
       </c>
       <c r="H116" s="5" t="n">
-        <v>-0.08270676691729323</v>
+        <v>-0.03692201518288475</v>
       </c>
       <c r="I116" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J116" s="5" t="n">
-        <v>-0.08247442764521856</v>
+        <v>-0.03668967591081009</v>
       </c>
     </row>
     <row r="117">
@@ -7013,34 +7013,34 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>6727</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>ワコム</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F117" s="4" t="n">
-        <v>880</v>
+        <v>2898</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>863</v>
+        <v>2809</v>
       </c>
       <c r="H117" s="5" t="n">
-        <v>-0.01931818181818182</v>
+        <v>-0.03071083505866114</v>
       </c>
       <c r="I117" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J117" s="5" t="n">
-        <v>-0.01908584254610715</v>
+        <v>-0.04465459562155183</v>
       </c>
     </row>
     <row r="118">
@@ -7049,12 +7049,12 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D118" s="2" t="n">
@@ -7064,19 +7064,19 @@
         <v>7</v>
       </c>
       <c r="F118" s="4" t="n">
-        <v>1544</v>
+        <v>2399</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>1466</v>
+        <v>2245</v>
       </c>
       <c r="H118" s="5" t="n">
-        <v>-0.05051813471502591</v>
+        <v>-0.06419341392246769</v>
       </c>
       <c r="I118" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J118" s="5" t="n">
-        <v>-0.05028579544295124</v>
+        <v>-0.06396107465039302</v>
       </c>
     </row>
     <row r="119">
@@ -7085,34 +7085,34 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>4503</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F119" s="4" t="n">
-        <v>1295</v>
+        <v>2399</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>1209</v>
+        <v>2235</v>
       </c>
       <c r="H119" s="5" t="n">
-        <v>-0.06640926640926641</v>
+        <v>-0.06836181742392664</v>
       </c>
       <c r="I119" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>0.01394376056289069</v>
       </c>
       <c r="J119" s="5" t="n">
-        <v>-0.06617692713719174</v>
+        <v>-0.08230557798681733</v>
       </c>
     </row>
     <row r="120">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>8624</t>
+          <t>5101</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>いちよし証券</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="D120" s="2" t="n">
@@ -7136,19 +7136,19 @@
         <v>7</v>
       </c>
       <c r="F120" s="4" t="n">
-        <v>1710</v>
+        <v>6986</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>1601</v>
+        <v>7061</v>
       </c>
       <c r="H120" s="5" t="n">
-        <v>-0.06374269005847953</v>
+        <v>0.0107357572287432</v>
       </c>
       <c r="I120" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
       <c r="J120" s="5" t="n">
-        <v>-0.06351035078640486</v>
+        <v>0.01096809650081787</v>
       </c>
     </row>
     <row r="121">
@@ -7157,34 +7157,754 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
+          <t>5101</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>横浜ゴム</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E121" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F121" s="4" t="n">
+        <v>6986</v>
+      </c>
+      <c r="G121" s="4" t="n">
+        <v>7191</v>
+      </c>
+      <c r="H121" s="5" t="n">
+        <v>0.02934440309189808</v>
+      </c>
+      <c r="I121" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J121" s="5" t="n">
+        <v>0.01540064252900739</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E122" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F122" s="4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="G122" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="H122" s="5" t="n">
+        <v>-0.03047091412742382</v>
+      </c>
+      <c r="I122" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J122" s="5" t="n">
+        <v>-0.03023857485534916</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E123" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F123" s="4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="G123" s="4" t="n">
+        <v>2484</v>
+      </c>
+      <c r="H123" s="5" t="n">
+        <v>-0.01701622477245746</v>
+      </c>
+      <c r="I123" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J123" s="5" t="n">
+        <v>-0.03095998533534815</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>5445</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>東京鐵鋼</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E124" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F124" s="4" t="n">
+        <v>2067</v>
+      </c>
+      <c r="G124" s="4" t="n">
+        <v>1950</v>
+      </c>
+      <c r="H124" s="5" t="n">
+        <v>-0.05660377358490566</v>
+      </c>
+      <c r="I124" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J124" s="5" t="n">
+        <v>-0.056371434312831</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>5445</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>東京鐵鋼</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E125" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F125" s="4" t="n">
+        <v>2067</v>
+      </c>
+      <c r="G125" s="4" t="n">
+        <v>1926</v>
+      </c>
+      <c r="H125" s="5" t="n">
+        <v>-0.06821480406386067</v>
+      </c>
+      <c r="I125" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J125" s="5" t="n">
+        <v>-0.08215856462675136</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E126" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F126" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="G126" s="4" t="n">
+        <v>2553.5</v>
+      </c>
+      <c r="H126" s="5" t="n">
+        <v>-0.8888574537540805</v>
+      </c>
+      <c r="I126" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J126" s="5" t="n">
+        <v>-0.8886251144820059</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>5706</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>三井金属</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E127" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F127" s="4" t="n">
+        <v>22975</v>
+      </c>
+      <c r="G127" s="4" t="n">
+        <v>2647.5</v>
+      </c>
+      <c r="H127" s="5" t="n">
+        <v>-0.884766050054407</v>
+      </c>
+      <c r="I127" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>-0.8987098106172977</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E128" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F128" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="G128" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="H128" s="5" t="n">
+        <v>-0.007407407407407408</v>
+      </c>
+      <c r="I128" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J128" s="5" t="n">
+        <v>-0.00717506813533274</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E129" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F129" s="4" t="n">
+        <v>675</v>
+      </c>
+      <c r="G129" s="4" t="n">
+        <v>660</v>
+      </c>
+      <c r="H129" s="5" t="n">
+        <v>-0.02222222222222222</v>
+      </c>
+      <c r="I129" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J129" s="5" t="n">
+        <v>-0.03616598278511291</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E130" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F130" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="G130" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="H130" s="5" t="n">
+        <v>-0.08270676691729323</v>
+      </c>
+      <c r="I130" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J130" s="5" t="n">
+        <v>-0.08247442764521856</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E131" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F131" s="4" t="n">
+        <v>3325</v>
+      </c>
+      <c r="G131" s="4" t="n">
+        <v>3045</v>
+      </c>
+      <c r="H131" s="5" t="n">
+        <v>-0.08421052631578947</v>
+      </c>
+      <c r="I131" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J131" s="5" t="n">
+        <v>-0.09815428687868016</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E132" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F132" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="G132" s="4" t="n">
+        <v>863</v>
+      </c>
+      <c r="H132" s="5" t="n">
+        <v>-0.01931818181818182</v>
+      </c>
+      <c r="I132" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J132" s="5" t="n">
+        <v>-0.01908584254610715</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E133" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F133" s="4" t="n">
+        <v>880</v>
+      </c>
+      <c r="G133" s="4" t="n">
+        <v>892</v>
+      </c>
+      <c r="H133" s="5" t="n">
+        <v>0.01363636363636364</v>
+      </c>
+      <c r="I133" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>-0.0003073969265270527</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E134" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F134" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="G134" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="H134" s="5" t="n">
+        <v>-0.05051813471502591</v>
+      </c>
+      <c r="I134" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J134" s="5" t="n">
+        <v>-0.05028579544295124</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E135" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F135" s="4" t="n">
+        <v>1544</v>
+      </c>
+      <c r="G135" s="4" t="n">
+        <v>1490</v>
+      </c>
+      <c r="H135" s="5" t="n">
+        <v>-0.0349740932642487</v>
+      </c>
+      <c r="I135" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>-0.0489178538271394</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E136" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F136" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="G136" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="H136" s="5" t="n">
+        <v>-0.06640926640926641</v>
+      </c>
+      <c r="I136" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J136" s="5" t="n">
+        <v>-0.06617692713719174</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E137" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F137" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="G137" s="4" t="n">
+        <v>1210</v>
+      </c>
+      <c r="H137" s="5" t="n">
+        <v>-0.06563706563706563</v>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>-0.07958082619995632</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F138" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G138" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="H138" s="5" t="n">
+        <v>-0.06374269005847953</v>
+      </c>
+      <c r="I138" s="5" t="n">
+        <v>-0.000232339272074667</v>
+      </c>
+      <c r="J138" s="5" t="n">
+        <v>-0.06351035078640486</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E139" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F139" s="4" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G139" s="4" t="n">
+        <v>1627</v>
+      </c>
+      <c r="H139" s="5" t="n">
+        <v>-0.04853801169590644</v>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>-0.06248177225879713</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
           <t>9757</t>
         </is>
       </c>
-      <c r="C121" s="3" t="inlineStr">
+      <c r="C140" s="3" t="inlineStr">
         <is>
           <t>船井総研ホールディングス</t>
         </is>
       </c>
-      <c r="D121" s="2" t="n">
+      <c r="D140" s="2" t="n">
         <v>46298</v>
       </c>
-      <c r="E121" s="3" t="n">
+      <c r="E140" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F121" s="4" t="n">
+      <c r="F140" s="4" t="n">
         <v>1191</v>
       </c>
-      <c r="G121" s="4" t="n">
+      <c r="G140" s="4" t="n">
         <v>1165</v>
       </c>
-      <c r="H121" s="5" t="n">
+      <c r="H140" s="5" t="n">
         <v>-0.0218303946263644</v>
       </c>
-      <c r="I121" s="5" t="n">
+      <c r="I140" s="5" t="n">
         <v>-0.000232339272074667</v>
       </c>
-      <c r="J121" s="5" t="n">
+      <c r="J140" s="5" t="n">
         <v>-0.02159805535428973</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E141" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F141" s="4" t="n">
+        <v>1191</v>
+      </c>
+      <c r="G141" s="4" t="n">
+        <v>1158</v>
+      </c>
+      <c r="H141" s="5" t="n">
+        <v>-0.02770780856423174</v>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>0.01394376056289069</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>-0.04165156912712242</v>
       </c>
     </row>
   </sheetData>
@@ -7942,7 +8662,9 @@
       <c r="H22" s="4" t="n">
         <v>2119</v>
       </c>
-      <c r="I22" s="4" t="n"/>
+      <c r="I22" s="4" t="n">
+        <v>2125</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -7967,7 +8689,9 @@
       <c r="H23" s="4" t="n">
         <v>424</v>
       </c>
-      <c r="I23" s="4" t="n"/>
+      <c r="I23" s="4" t="n">
+        <v>422</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -7992,7 +8716,9 @@
       <c r="H24" s="4" t="n">
         <v>3370</v>
       </c>
-      <c r="I24" s="4" t="n"/>
+      <c r="I24" s="4" t="n">
+        <v>3360</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -8017,7 +8743,9 @@
       <c r="H25" s="4" t="n">
         <v>2345</v>
       </c>
-      <c r="I25" s="4" t="n"/>
+      <c r="I25" s="4" t="n">
+        <v>2362</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -8042,7 +8770,9 @@
       <c r="H26" s="4" t="n">
         <v>1645.5</v>
       </c>
-      <c r="I26" s="4" t="n"/>
+      <c r="I26" s="4" t="n">
+        <v>1620.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -8067,7 +8797,9 @@
       <c r="H27" s="4" t="n">
         <v>4710</v>
       </c>
-      <c r="I27" s="4" t="n"/>
+      <c r="I27" s="4" t="n">
+        <v>4655</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -8092,7 +8824,9 @@
       <c r="H28" s="4" t="n">
         <v>2038</v>
       </c>
-      <c r="I28" s="4" t="n"/>
+      <c r="I28" s="4" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -8117,7 +8851,9 @@
       <c r="H29" s="4" t="n">
         <v>2791</v>
       </c>
-      <c r="I29" s="4" t="n"/>
+      <c r="I29" s="4" t="n">
+        <v>2809</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -8142,7 +8878,9 @@
       <c r="H30" s="4" t="n">
         <v>2245</v>
       </c>
-      <c r="I30" s="4" t="n"/>
+      <c r="I30" s="4" t="n">
+        <v>2235</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -8167,7 +8905,9 @@
       <c r="H31" s="4" t="n">
         <v>7061</v>
       </c>
-      <c r="I31" s="4" t="n"/>
+      <c r="I31" s="4" t="n">
+        <v>7191</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -8192,7 +8932,9 @@
       <c r="H32" s="4" t="n">
         <v>2450</v>
       </c>
-      <c r="I32" s="4" t="n"/>
+      <c r="I32" s="4" t="n">
+        <v>2484</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -8217,7 +8959,9 @@
       <c r="H33" s="4" t="n">
         <v>1950</v>
       </c>
-      <c r="I33" s="4" t="n"/>
+      <c r="I33" s="4" t="n">
+        <v>1926</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -8242,7 +8986,9 @@
       <c r="H34" s="4" t="n">
         <v>2553.5</v>
       </c>
-      <c r="I34" s="4" t="n"/>
+      <c r="I34" s="4" t="n">
+        <v>2647.5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -8267,7 +9013,9 @@
       <c r="H35" s="4" t="n">
         <v>670</v>
       </c>
-      <c r="I35" s="4" t="n"/>
+      <c r="I35" s="4" t="n">
+        <v>660</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -8292,7 +9040,9 @@
       <c r="H36" s="4" t="n">
         <v>3050</v>
       </c>
-      <c r="I36" s="4" t="n"/>
+      <c r="I36" s="4" t="n">
+        <v>3045</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -8317,7 +9067,9 @@
       <c r="H37" s="4" t="n">
         <v>863</v>
       </c>
-      <c r="I37" s="4" t="n"/>
+      <c r="I37" s="4" t="n">
+        <v>892</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -8342,7 +9094,9 @@
       <c r="H38" s="4" t="n">
         <v>1466</v>
       </c>
-      <c r="I38" s="4" t="n"/>
+      <c r="I38" s="4" t="n">
+        <v>1490</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -8367,7 +9121,9 @@
       <c r="H39" s="4" t="n">
         <v>1209</v>
       </c>
-      <c r="I39" s="4" t="n"/>
+      <c r="I39" s="4" t="n">
+        <v>1210</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -8392,7 +9148,9 @@
       <c r="H40" s="4" t="n">
         <v>1601</v>
       </c>
-      <c r="I40" s="4" t="n"/>
+      <c r="I40" s="4" t="n">
+        <v>1627</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -8417,7 +9175,9 @@
       <c r="H41" s="4" t="n">
         <v>1165</v>
       </c>
-      <c r="I41" s="4" t="n"/>
+      <c r="I41" s="4" t="n">
+        <v>1158</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">

</xml_diff>

<commit_message>
Performance check 2026-10-03 -> 2026-10-05
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -2800,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7905,6 +7905,726 @@
       </c>
       <c r="J141" s="5" t="n">
         <v>-0.04165156912712242</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>1926</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>ライト工業</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F142" s="4" t="n">
+        <v>952</v>
+      </c>
+      <c r="G142" s="4" t="n">
+        <v>950</v>
+      </c>
+      <c r="H142" s="5" t="n">
+        <v>-0.002100840336134454</v>
+      </c>
+      <c r="I142" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J142" s="5" t="n">
+        <v>-0.01628023460124169</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E143" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F143" s="4" t="n">
+        <v>3835</v>
+      </c>
+      <c r="G143" s="4" t="n">
+        <v>3870</v>
+      </c>
+      <c r="H143" s="5" t="n">
+        <v>0.009126466753585397</v>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>-0.005052927511521839</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F144" s="4" t="n">
+        <v>2119</v>
+      </c>
+      <c r="G144" s="4" t="n">
+        <v>2125</v>
+      </c>
+      <c r="H144" s="5" t="n">
+        <v>0.002831524303916942</v>
+      </c>
+      <c r="I144" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J144" s="5" t="n">
+        <v>-0.01134786996119029</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E145" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F145" s="4" t="n">
+        <v>424</v>
+      </c>
+      <c r="G145" s="4" t="n">
+        <v>422</v>
+      </c>
+      <c r="H145" s="5" t="n">
+        <v>-0.004716981132075472</v>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>-0.01889637539718271</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F146" s="4" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G146" s="4" t="n">
+        <v>3360</v>
+      </c>
+      <c r="H146" s="5" t="n">
+        <v>-0.002967359050445104</v>
+      </c>
+      <c r="I146" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J146" s="5" t="n">
+        <v>-0.01714675331555234</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E147" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F147" s="4" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G147" s="4" t="n">
+        <v>2362</v>
+      </c>
+      <c r="H147" s="5" t="n">
+        <v>0.007249466950959489</v>
+      </c>
+      <c r="I147" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J147" s="5" t="n">
+        <v>-0.006929927314147748</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F148" s="4" t="n">
+        <v>1645.5</v>
+      </c>
+      <c r="G148" s="4" t="n">
+        <v>1620.5</v>
+      </c>
+      <c r="H148" s="5" t="n">
+        <v>-0.01519295047098146</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J148" s="5" t="n">
+        <v>-0.0293723447360887</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F149" s="4" t="n">
+        <v>4710</v>
+      </c>
+      <c r="G149" s="4" t="n">
+        <v>4655</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>-0.01167728237791932</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J149" s="5" t="n">
+        <v>-0.02585667664302656</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F150" s="4" t="n">
+        <v>2038</v>
+      </c>
+      <c r="G150" s="4" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H150" s="5" t="n">
+        <v>-0.007850834151128557</v>
+      </c>
+      <c r="I150" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J150" s="5" t="n">
+        <v>-0.02203022841623579</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E151" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F151" s="4" t="n">
+        <v>2791</v>
+      </c>
+      <c r="G151" s="4" t="n">
+        <v>2809</v>
+      </c>
+      <c r="H151" s="5" t="n">
+        <v>0.006449301325689717</v>
+      </c>
+      <c r="I151" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J151" s="5" t="n">
+        <v>-0.00773009293941752</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F152" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="G152" s="4" t="n">
+        <v>2235</v>
+      </c>
+      <c r="H152" s="5" t="n">
+        <v>-0.004454342984409799</v>
+      </c>
+      <c r="I152" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J152" s="5" t="n">
+        <v>-0.01863373724951704</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E153" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F153" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G153" s="4" t="n">
+        <v>2484</v>
+      </c>
+      <c r="H153" s="5" t="n">
+        <v>0.01387755102040816</v>
+      </c>
+      <c r="I153" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J153" s="5" t="n">
+        <v>-0.0003018432446990731</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F154" s="4" t="n">
+        <v>3758</v>
+      </c>
+      <c r="G154" s="4" t="n">
+        <v>3947</v>
+      </c>
+      <c r="H154" s="5" t="n">
+        <v>0.05029270888770623</v>
+      </c>
+      <c r="I154" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J154" s="5" t="n">
+        <v>0.03611331462259899</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E155" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F155" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="G155" s="4" t="n">
+        <v>660</v>
+      </c>
+      <c r="H155" s="5" t="n">
+        <v>-0.01492537313432836</v>
+      </c>
+      <c r="I155" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J155" s="5" t="n">
+        <v>-0.02910476739943559</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F156" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G156" s="4" t="n">
+        <v>3045</v>
+      </c>
+      <c r="H156" s="5" t="n">
+        <v>-0.001639344262295082</v>
+      </c>
+      <c r="I156" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J156" s="5" t="n">
+        <v>-0.01581873852740232</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E157" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F157" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="G157" s="4" t="n">
+        <v>1490</v>
+      </c>
+      <c r="H157" s="5" t="n">
+        <v>0.01637107776261937</v>
+      </c>
+      <c r="I157" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J157" s="5" t="n">
+        <v>0.002191683497512135</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F158" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="G158" s="4" t="n">
+        <v>1210</v>
+      </c>
+      <c r="H158" s="5" t="n">
+        <v>0.0008271298593879239</v>
+      </c>
+      <c r="I158" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J158" s="5" t="n">
+        <v>-0.01335226440571931</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>東京エレクトロン</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E159" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F159" s="4" t="n">
+        <v>12100</v>
+      </c>
+      <c r="G159" s="4" t="n">
+        <v>12765</v>
+      </c>
+      <c r="H159" s="5" t="n">
+        <v>0.05495867768595041</v>
+      </c>
+      <c r="I159" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J159" s="5" t="n">
+        <v>0.04077928342084318</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F160" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="G160" s="4" t="n">
+        <v>1627</v>
+      </c>
+      <c r="H160" s="5" t="n">
+        <v>0.01623985009369144</v>
+      </c>
+      <c r="I160" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J160" s="5" t="n">
+        <v>0.002060455828584207</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E161" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F161" s="4" t="n">
+        <v>1165</v>
+      </c>
+      <c r="G161" s="4" t="n">
+        <v>1158</v>
+      </c>
+      <c r="H161" s="5" t="n">
+        <v>-0.006008583690987125</v>
+      </c>
+      <c r="I161" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J161" s="5" t="n">
+        <v>-0.02018797795609436</v>
       </c>
     </row>
   </sheetData>
@@ -9200,7 +9920,9 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
       <c r="H42" s="4" t="n"/>
-      <c r="I42" s="4" t="n"/>
+      <c r="I42" s="4" t="n">
+        <v>950</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -9223,7 +9945,9 @@
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
       <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
+      <c r="I43" s="4" t="n">
+        <v>3870</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -9246,7 +9970,9 @@
       <c r="F44" s="4" t="n"/>
       <c r="G44" s="4" t="n"/>
       <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
+      <c r="I44" s="4" t="n">
+        <v>2125</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -9269,7 +9995,9 @@
       <c r="F45" s="4" t="n"/>
       <c r="G45" s="4" t="n"/>
       <c r="H45" s="4" t="n"/>
-      <c r="I45" s="4" t="n"/>
+      <c r="I45" s="4" t="n">
+        <v>422</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -9292,7 +10020,9 @@
       <c r="F46" s="4" t="n"/>
       <c r="G46" s="4" t="n"/>
       <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
+      <c r="I46" s="4" t="n">
+        <v>3360</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -9315,7 +10045,9 @@
       <c r="F47" s="4" t="n"/>
       <c r="G47" s="4" t="n"/>
       <c r="H47" s="4" t="n"/>
-      <c r="I47" s="4" t="n"/>
+      <c r="I47" s="4" t="n">
+        <v>2362</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -9338,7 +10070,9 @@
       <c r="F48" s="4" t="n"/>
       <c r="G48" s="4" t="n"/>
       <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
+      <c r="I48" s="4" t="n">
+        <v>1620.5</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -9361,7 +10095,9 @@
       <c r="F49" s="4" t="n"/>
       <c r="G49" s="4" t="n"/>
       <c r="H49" s="4" t="n"/>
-      <c r="I49" s="4" t="n"/>
+      <c r="I49" s="4" t="n">
+        <v>4655</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -9384,7 +10120,9 @@
       <c r="F50" s="4" t="n"/>
       <c r="G50" s="4" t="n"/>
       <c r="H50" s="4" t="n"/>
-      <c r="I50" s="4" t="n"/>
+      <c r="I50" s="4" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -9407,7 +10145,9 @@
       <c r="F51" s="4" t="n"/>
       <c r="G51" s="4" t="n"/>
       <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
+      <c r="I51" s="4" t="n">
+        <v>2809</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -9430,7 +10170,9 @@
       <c r="F52" s="4" t="n"/>
       <c r="G52" s="4" t="n"/>
       <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
+      <c r="I52" s="4" t="n">
+        <v>2235</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -9453,7 +10195,9 @@
       <c r="F53" s="4" t="n"/>
       <c r="G53" s="4" t="n"/>
       <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="n"/>
+      <c r="I53" s="4" t="n">
+        <v>2484</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -9476,7 +10220,9 @@
       <c r="F54" s="4" t="n"/>
       <c r="G54" s="4" t="n"/>
       <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
+      <c r="I54" s="4" t="n">
+        <v>3947</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -9499,7 +10245,9 @@
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
       <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
+      <c r="I55" s="4" t="n">
+        <v>660</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -9522,7 +10270,9 @@
       <c r="F56" s="4" t="n"/>
       <c r="G56" s="4" t="n"/>
       <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
+      <c r="I56" s="4" t="n">
+        <v>3045</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -9545,7 +10295,9 @@
       <c r="F57" s="4" t="n"/>
       <c r="G57" s="4" t="n"/>
       <c r="H57" s="4" t="n"/>
-      <c r="I57" s="4" t="n"/>
+      <c r="I57" s="4" t="n">
+        <v>1490</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -9568,7 +10320,9 @@
       <c r="F58" s="4" t="n"/>
       <c r="G58" s="4" t="n"/>
       <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
+      <c r="I58" s="4" t="n">
+        <v>1210</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -9591,7 +10345,9 @@
       <c r="F59" s="4" t="n"/>
       <c r="G59" s="4" t="n"/>
       <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
+      <c r="I59" s="4" t="n">
+        <v>12765</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -9614,7 +10370,9 @@
       <c r="F60" s="4" t="n"/>
       <c r="G60" s="4" t="n"/>
       <c r="H60" s="4" t="n"/>
-      <c r="I60" s="4" t="n"/>
+      <c r="I60" s="4" t="n">
+        <v>1627</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -9637,7 +10395,9 @@
       <c r="F61" s="4" t="n"/>
       <c r="G61" s="4" t="n"/>
       <c r="H61" s="4" t="n"/>
-      <c r="I61" s="4" t="n"/>
+      <c r="I61" s="4" t="n">
+        <v>1158</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record entry prices 2026-10-10
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週次ピック" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="価格推移ログ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="価格推移(ピボット)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="週次ピック" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="価格推移ログ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="価格推移(ピボット)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2787,6 +2787,766 @@
       </c>
       <c r="J61" s="4" t="n">
         <v>430.2000122070313</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>3932</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>アカツキ</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>証券、商品先物取引業</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>1561</v>
+      </c>
+      <c r="J63" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="I64" s="4" t="n">
+        <v>3828</v>
+      </c>
+      <c r="J64" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>電気・ガス業</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>2389</v>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>食料品</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>2157</v>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="I67" s="4" t="n">
+        <v>2918</v>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>3415</v>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>医薬品</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="I69" s="4" t="n">
+        <v>2247.5</v>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>1637</v>
+      </c>
+      <c r="J70" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>695</v>
+      </c>
+      <c r="J71" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>97.2</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>1134</v>
+      </c>
+      <c r="J72" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>輸送用機器</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>1431</v>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>433</v>
+      </c>
+      <c r="J74" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>4745</v>
+      </c>
+      <c r="J75" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I76" s="4" t="n">
+        <v>1241</v>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="I77" s="4" t="n">
+        <v>2814</v>
+      </c>
+      <c r="J77" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="I78" s="4" t="n">
+        <v>2133</v>
+      </c>
+      <c r="J78" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="H79" s="3" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="I79" s="4" t="n">
+        <v>2485</v>
+      </c>
+      <c r="J79" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="H80" s="3" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="I80" s="4" t="n">
+        <v>3845</v>
+      </c>
+      <c r="J80" s="4" t="n">
+        <v>432.5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="H81" s="3" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>1978</v>
+      </c>
+      <c r="J81" s="4" t="n">
+        <v>432.5</v>
       </c>
     </row>
   </sheetData>
@@ -8638,7 +9398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10399,6 +11159,466 @@
         <v>1158</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>3845</v>
+      </c>
+      <c r="E62" s="4" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n">
+        <v>2157</v>
+      </c>
+      <c r="E63" s="4" t="n"/>
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n">
+        <v>433</v>
+      </c>
+      <c r="E64" s="4" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
+      <c r="I64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="n">
+        <v>3415</v>
+      </c>
+      <c r="E65" s="4" t="n"/>
+      <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
+      <c r="I65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="n">
+        <v>2389</v>
+      </c>
+      <c r="E66" s="4" t="n"/>
+      <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="n">
+        <v>1637</v>
+      </c>
+      <c r="E67" s="4" t="n"/>
+      <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
+      <c r="I67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="n">
+        <v>4745</v>
+      </c>
+      <c r="E68" s="4" t="n"/>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="n">
+        <v>2133</v>
+      </c>
+      <c r="E69" s="4" t="n"/>
+      <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
+      <c r="I69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="n">
+        <v>1134</v>
+      </c>
+      <c r="E70" s="4" t="n"/>
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
+      <c r="I70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>3932</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>アカツキ</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="E71" s="4" t="n"/>
+      <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n">
+        <v>2814</v>
+      </c>
+      <c r="E72" s="4" t="n"/>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
+      <c r="I72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="n">
+        <v>2247.5</v>
+      </c>
+      <c r="E73" s="4" t="n"/>
+      <c r="F73" s="4" t="n"/>
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
+      <c r="I73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n">
+        <v>2485</v>
+      </c>
+      <c r="E74" s="4" t="n"/>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
+      <c r="I74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="n">
+        <v>3828</v>
+      </c>
+      <c r="E75" s="4" t="n"/>
+      <c r="F75" s="4" t="n"/>
+      <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n">
+        <v>695</v>
+      </c>
+      <c r="E76" s="4" t="n"/>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="n">
+        <v>2918</v>
+      </c>
+      <c r="E77" s="4" t="n"/>
+      <c r="F77" s="4" t="n"/>
+      <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
+      <c r="I77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="n">
+        <v>1978</v>
+      </c>
+      <c r="E78" s="4" t="n"/>
+      <c r="F78" s="4" t="n"/>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="n">
+        <v>1431</v>
+      </c>
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>1241</v>
+      </c>
+      <c r="E80" s="4" t="n"/>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="n">
+        <v>1561</v>
+      </c>
+      <c r="E81" s="4" t="n"/>
+      <c r="F81" s="4" t="n"/>
+      <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
+      <c r="I81" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Performance check 2026-10-03 -> 2026-10-10
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -3560,7 +3560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8709,34 +8709,34 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1926</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>朝日工業社</t>
+          <t>ライト工業</t>
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F143" s="4" t="n">
-        <v>3835</v>
+        <v>952</v>
       </c>
       <c r="G143" s="4" t="n">
-        <v>3870</v>
+        <v>935</v>
       </c>
       <c r="H143" s="5" t="n">
-        <v>0.009126466753585397</v>
+        <v>-0.01785714285714286</v>
       </c>
       <c r="I143" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J143" s="5" t="n">
-        <v>-0.005052927511521839</v>
+        <v>-0.02320346486482759</v>
       </c>
     </row>
     <row r="144">
@@ -8745,12 +8745,12 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>2288</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>丸大食品</t>
+          <t>朝日工業社</t>
         </is>
       </c>
       <c r="D144" s="2" t="n">
@@ -8760,19 +8760,19 @@
         <v>2</v>
       </c>
       <c r="F144" s="4" t="n">
-        <v>2119</v>
+        <v>3835</v>
       </c>
       <c r="G144" s="4" t="n">
-        <v>2125</v>
+        <v>3870</v>
       </c>
       <c r="H144" s="5" t="n">
-        <v>0.002831524303916942</v>
+        <v>0.009126466753585397</v>
       </c>
       <c r="I144" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J144" s="5" t="n">
-        <v>-0.01134786996119029</v>
+        <v>-0.005052927511521839</v>
       </c>
     </row>
     <row r="145">
@@ -8781,34 +8781,34 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>システナ</t>
+          <t>朝日工業社</t>
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F145" s="4" t="n">
-        <v>424</v>
+        <v>3835</v>
       </c>
       <c r="G145" s="4" t="n">
-        <v>422</v>
+        <v>3845</v>
       </c>
       <c r="H145" s="5" t="n">
-        <v>-0.004716981132075472</v>
+        <v>0.002607561929595828</v>
       </c>
       <c r="I145" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J145" s="5" t="n">
-        <v>-0.01889637539718271</v>
+        <v>-0.002738760078088908</v>
       </c>
     </row>
     <row r="146">
@@ -8817,12 +8817,12 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>3110</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>日東紡績</t>
+          <t>丸大食品</t>
         </is>
       </c>
       <c r="D146" s="2" t="n">
@@ -8832,19 +8832,19 @@
         <v>2</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>3370</v>
+        <v>2119</v>
       </c>
       <c r="G146" s="4" t="n">
-        <v>3360</v>
+        <v>2125</v>
       </c>
       <c r="H146" s="5" t="n">
-        <v>-0.002967359050445104</v>
+        <v>0.002831524303916942</v>
       </c>
       <c r="I146" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J146" s="5" t="n">
-        <v>-0.01714675331555234</v>
+        <v>-0.01134786996119029</v>
       </c>
     </row>
     <row r="147">
@@ -8853,34 +8853,34 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>3150</t>
+          <t>2288</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>グリムス</t>
+          <t>丸大食品</t>
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E147" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F147" s="4" t="n">
-        <v>2345</v>
+        <v>2119</v>
       </c>
       <c r="G147" s="4" t="n">
-        <v>2362</v>
+        <v>2157</v>
       </c>
       <c r="H147" s="5" t="n">
-        <v>0.007249466950959489</v>
+        <v>0.01793298725814063</v>
       </c>
       <c r="I147" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J147" s="5" t="n">
-        <v>-0.006929927314147748</v>
+        <v>0.0125866652504559</v>
       </c>
     </row>
     <row r="148">
@@ -8889,12 +8889,12 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>3635</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>コーエーテクモホールディングス</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D148" s="2" t="n">
@@ -8904,19 +8904,19 @@
         <v>2</v>
       </c>
       <c r="F148" s="4" t="n">
-        <v>1645.5</v>
+        <v>424</v>
       </c>
       <c r="G148" s="4" t="n">
-        <v>1620.5</v>
+        <v>422</v>
       </c>
       <c r="H148" s="5" t="n">
-        <v>-0.01519295047098146</v>
+        <v>-0.004716981132075472</v>
       </c>
       <c r="I148" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J148" s="5" t="n">
-        <v>-0.0293723447360887</v>
+        <v>-0.01889637539718271</v>
       </c>
     </row>
     <row r="149">
@@ -8925,34 +8925,34 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>3817</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>ＳＲＡホールディングス</t>
+          <t>システナ</t>
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E149" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F149" s="4" t="n">
-        <v>4710</v>
+        <v>424</v>
       </c>
       <c r="G149" s="4" t="n">
-        <v>4655</v>
+        <v>433</v>
       </c>
       <c r="H149" s="5" t="n">
-        <v>-0.01167728237791932</v>
+        <v>0.02122641509433962</v>
       </c>
       <c r="I149" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J149" s="5" t="n">
-        <v>-0.02585667664302656</v>
+        <v>0.01588009308665489</v>
       </c>
     </row>
     <row r="150">
@@ -8961,12 +8961,12 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>3854</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>アイル</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D150" s="2" t="n">
@@ -8976,19 +8976,19 @@
         <v>2</v>
       </c>
       <c r="F150" s="4" t="n">
-        <v>2038</v>
+        <v>3370</v>
       </c>
       <c r="G150" s="4" t="n">
-        <v>2022</v>
+        <v>3360</v>
       </c>
       <c r="H150" s="5" t="n">
-        <v>-0.007850834151128557</v>
+        <v>-0.002967359050445104</v>
       </c>
       <c r="I150" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J150" s="5" t="n">
-        <v>-0.02203022841623579</v>
+        <v>-0.01714675331555234</v>
       </c>
     </row>
     <row r="151">
@@ -8997,34 +8997,34 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>4028</t>
+          <t>3110</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>石原産業</t>
+          <t>日東紡績</t>
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E151" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F151" s="4" t="n">
-        <v>2791</v>
+        <v>3370</v>
       </c>
       <c r="G151" s="4" t="n">
-        <v>2809</v>
+        <v>3415</v>
       </c>
       <c r="H151" s="5" t="n">
-        <v>0.006449301325689717</v>
+        <v>0.01335311572700297</v>
       </c>
       <c r="I151" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J151" s="5" t="n">
-        <v>-0.00773009293941752</v>
+        <v>0.008006793719318232</v>
       </c>
     </row>
     <row r="152">
@@ -9033,12 +9033,12 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>4503</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>アステラス製薬</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D152" s="2" t="n">
@@ -9048,19 +9048,19 @@
         <v>2</v>
       </c>
       <c r="F152" s="4" t="n">
-        <v>2245</v>
+        <v>2345</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>2235</v>
+        <v>2362</v>
       </c>
       <c r="H152" s="5" t="n">
-        <v>-0.004454342984409799</v>
+        <v>0.007249466950959489</v>
       </c>
       <c r="I152" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J152" s="5" t="n">
-        <v>-0.01863373724951704</v>
+        <v>-0.006929927314147748</v>
       </c>
     </row>
     <row r="153">
@@ -9069,34 +9069,34 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>5195</t>
+          <t>3150</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>バンドー化学</t>
+          <t>グリムス</t>
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E153" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F153" s="4" t="n">
-        <v>2450</v>
+        <v>2345</v>
       </c>
       <c r="G153" s="4" t="n">
-        <v>2484</v>
+        <v>2389</v>
       </c>
       <c r="H153" s="5" t="n">
-        <v>0.01387755102040816</v>
+        <v>0.01876332622601279</v>
       </c>
       <c r="I153" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J153" s="5" t="n">
-        <v>-0.0003018432446990731</v>
+        <v>0.01341700421832806</v>
       </c>
     </row>
     <row r="154">
@@ -9105,12 +9105,12 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>5334</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>日本特殊陶業</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D154" s="2" t="n">
@@ -9120,19 +9120,19 @@
         <v>2</v>
       </c>
       <c r="F154" s="4" t="n">
-        <v>3758</v>
+        <v>1645.5</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>3947</v>
+        <v>1620.5</v>
       </c>
       <c r="H154" s="5" t="n">
-        <v>0.05029270888770623</v>
+        <v>-0.01519295047098146</v>
       </c>
       <c r="I154" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J154" s="5" t="n">
-        <v>0.03611331462259899</v>
+        <v>-0.0293723447360887</v>
       </c>
     </row>
     <row r="155">
@@ -9141,34 +9141,34 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>6200</t>
+          <t>3635</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>インソース</t>
+          <t>コーエーテクモホールディングス</t>
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E155" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F155" s="4" t="n">
-        <v>670</v>
+        <v>1645.5</v>
       </c>
       <c r="G155" s="4" t="n">
-        <v>660</v>
+        <v>1637</v>
       </c>
       <c r="H155" s="5" t="n">
-        <v>-0.01492537313432836</v>
+        <v>-0.005165603160133698</v>
       </c>
       <c r="I155" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J155" s="5" t="n">
-        <v>-0.02910476739943559</v>
+        <v>-0.01051192516781843</v>
       </c>
     </row>
     <row r="156">
@@ -9177,12 +9177,12 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>6331</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>三菱化工機</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D156" s="2" t="n">
@@ -9192,19 +9192,19 @@
         <v>2</v>
       </c>
       <c r="F156" s="4" t="n">
-        <v>3050</v>
+        <v>4710</v>
       </c>
       <c r="G156" s="4" t="n">
-        <v>3045</v>
+        <v>4655</v>
       </c>
       <c r="H156" s="5" t="n">
-        <v>-0.001639344262295082</v>
+        <v>-0.01167728237791932</v>
       </c>
       <c r="I156" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J156" s="5" t="n">
-        <v>-0.01581873852740232</v>
+        <v>-0.02585667664302656</v>
       </c>
     </row>
     <row r="157">
@@ -9213,34 +9213,34 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>7236</t>
+          <t>3817</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>ティラド</t>
+          <t>ＳＲＡホールディングス</t>
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E157" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F157" s="4" t="n">
-        <v>1466</v>
+        <v>4710</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>1490</v>
+        <v>4745</v>
       </c>
       <c r="H157" s="5" t="n">
-        <v>0.01637107776261937</v>
+        <v>0.00743099787685775</v>
       </c>
       <c r="I157" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J157" s="5" t="n">
-        <v>0.002191683497512135</v>
+        <v>0.002084675869173014</v>
       </c>
     </row>
     <row r="158">
@@ -9249,12 +9249,12 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>7595</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>アルゴグラフィックス</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D158" s="2" t="n">
@@ -9264,19 +9264,19 @@
         <v>2</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>1209</v>
+        <v>2038</v>
       </c>
       <c r="G158" s="4" t="n">
-        <v>1210</v>
+        <v>2022</v>
       </c>
       <c r="H158" s="5" t="n">
-        <v>0.0008271298593879239</v>
+        <v>-0.007850834151128557</v>
       </c>
       <c r="I158" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J158" s="5" t="n">
-        <v>-0.01335226440571931</v>
+        <v>-0.02203022841623579</v>
       </c>
     </row>
     <row r="159">
@@ -9285,34 +9285,34 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>8035</t>
+          <t>3854</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>東京エレクトロン</t>
+          <t>アイル</t>
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>46300</v>
+        <v>46305</v>
       </c>
       <c r="E159" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>12100</v>
+        <v>2038</v>
       </c>
       <c r="G159" s="4" t="n">
-        <v>12765</v>
+        <v>2133</v>
       </c>
       <c r="H159" s="5" t="n">
-        <v>0.05495867768595041</v>
+        <v>0.04661432777232581</v>
       </c>
       <c r="I159" s="5" t="n">
-        <v>0.01417939426510724</v>
+        <v>0.005346322007684735</v>
       </c>
       <c r="J159" s="5" t="n">
-        <v>0.04077928342084318</v>
+        <v>0.04126800576464108</v>
       </c>
     </row>
     <row r="160">
@@ -9321,12 +9321,12 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>8624</t>
+          <t>4028</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>いちよし証券</t>
+          <t>石原産業</t>
         </is>
       </c>
       <c r="D160" s="2" t="n">
@@ -9336,19 +9336,19 @@
         <v>2</v>
       </c>
       <c r="F160" s="4" t="n">
-        <v>1601</v>
+        <v>2791</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>1627</v>
+        <v>2809</v>
       </c>
       <c r="H160" s="5" t="n">
-        <v>0.01623985009369144</v>
+        <v>0.006449301325689717</v>
       </c>
       <c r="I160" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
       <c r="J160" s="5" t="n">
-        <v>0.002060455828584207</v>
+        <v>-0.00773009293941752</v>
       </c>
     </row>
     <row r="161">
@@ -9357,34 +9357,754 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E161" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F161" s="4" t="n">
+        <v>2791</v>
+      </c>
+      <c r="G161" s="4" t="n">
+        <v>2814</v>
+      </c>
+      <c r="H161" s="5" t="n">
+        <v>0.008240773916159082</v>
+      </c>
+      <c r="I161" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J161" s="5" t="n">
+        <v>0.002894451908474347</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F162" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="G162" s="4" t="n">
+        <v>2235</v>
+      </c>
+      <c r="H162" s="5" t="n">
+        <v>-0.004454342984409799</v>
+      </c>
+      <c r="I162" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J162" s="5" t="n">
+        <v>-0.01863373724951704</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E163" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F163" s="4" t="n">
+        <v>2245</v>
+      </c>
+      <c r="G163" s="4" t="n">
+        <v>2247.5</v>
+      </c>
+      <c r="H163" s="5" t="n">
+        <v>0.00111358574610245</v>
+      </c>
+      <c r="I163" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J163" s="5" t="n">
+        <v>-0.004232736261582285</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E164" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F164" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G164" s="4" t="n">
+        <v>2484</v>
+      </c>
+      <c r="H164" s="5" t="n">
+        <v>0.01387755102040816</v>
+      </c>
+      <c r="I164" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J164" s="5" t="n">
+        <v>-0.0003018432446990731</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E165" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F165" s="4" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G165" s="4" t="n">
+        <v>2485</v>
+      </c>
+      <c r="H165" s="5" t="n">
+        <v>0.01428571428571429</v>
+      </c>
+      <c r="I165" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J165" s="5" t="n">
+        <v>0.00893939227802955</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E166" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F166" s="4" t="n">
+        <v>3758</v>
+      </c>
+      <c r="G166" s="4" t="n">
+        <v>3947</v>
+      </c>
+      <c r="H166" s="5" t="n">
+        <v>0.05029270888770623</v>
+      </c>
+      <c r="I166" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J166" s="5" t="n">
+        <v>0.03611331462259899</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E167" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F167" s="4" t="n">
+        <v>3758</v>
+      </c>
+      <c r="G167" s="4" t="n">
+        <v>3828</v>
+      </c>
+      <c r="H167" s="5" t="n">
+        <v>0.01862692921766897</v>
+      </c>
+      <c r="I167" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J167" s="5" t="n">
+        <v>0.01328060720998424</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E168" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F168" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="G168" s="4" t="n">
+        <v>660</v>
+      </c>
+      <c r="H168" s="5" t="n">
+        <v>-0.01492537313432836</v>
+      </c>
+      <c r="I168" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J168" s="5" t="n">
+        <v>-0.02910476739943559</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E169" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F169" s="4" t="n">
+        <v>670</v>
+      </c>
+      <c r="G169" s="4" t="n">
+        <v>695</v>
+      </c>
+      <c r="H169" s="5" t="n">
+        <v>0.03731343283582089</v>
+      </c>
+      <c r="I169" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J169" s="5" t="n">
+        <v>0.03196711082813616</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E170" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F170" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G170" s="4" t="n">
+        <v>3045</v>
+      </c>
+      <c r="H170" s="5" t="n">
+        <v>-0.001639344262295082</v>
+      </c>
+      <c r="I170" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J170" s="5" t="n">
+        <v>-0.01581873852740232</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E171" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F171" s="4" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G171" s="4" t="n">
+        <v>2918</v>
+      </c>
+      <c r="H171" s="5" t="n">
+        <v>-0.04327868852459017</v>
+      </c>
+      <c r="I171" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J171" s="5" t="n">
+        <v>-0.0486250105322749</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E172" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F172" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="G172" s="4" t="n">
+        <v>1490</v>
+      </c>
+      <c r="H172" s="5" t="n">
+        <v>0.01637107776261937</v>
+      </c>
+      <c r="I172" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J172" s="5" t="n">
+        <v>0.002191683497512135</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E173" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F173" s="4" t="n">
+        <v>1466</v>
+      </c>
+      <c r="G173" s="4" t="n">
+        <v>1431</v>
+      </c>
+      <c r="H173" s="5" t="n">
+        <v>-0.02387448840381992</v>
+      </c>
+      <c r="I173" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J173" s="5" t="n">
+        <v>-0.02922081041150465</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E174" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F174" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="G174" s="4" t="n">
+        <v>1210</v>
+      </c>
+      <c r="H174" s="5" t="n">
+        <v>0.0008271298593879239</v>
+      </c>
+      <c r="I174" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J174" s="5" t="n">
+        <v>-0.01335226440571931</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E175" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F175" s="4" t="n">
+        <v>1209</v>
+      </c>
+      <c r="G175" s="4" t="n">
+        <v>1241</v>
+      </c>
+      <c r="H175" s="5" t="n">
+        <v>0.02646815550041356</v>
+      </c>
+      <c r="I175" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J175" s="5" t="n">
+        <v>0.02112183349272883</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>東京エレクトロン</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E176" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F176" s="4" t="n">
+        <v>12100</v>
+      </c>
+      <c r="G176" s="4" t="n">
+        <v>12765</v>
+      </c>
+      <c r="H176" s="5" t="n">
+        <v>0.05495867768595041</v>
+      </c>
+      <c r="I176" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J176" s="5" t="n">
+        <v>0.04077928342084318</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>8035</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>東京エレクトロン</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E177" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F177" s="4" t="n">
+        <v>12100</v>
+      </c>
+      <c r="G177" s="4" t="n">
+        <v>12445</v>
+      </c>
+      <c r="H177" s="5" t="n">
+        <v>0.02851239669421488</v>
+      </c>
+      <c r="I177" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J177" s="5" t="n">
+        <v>0.02316607468653014</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E178" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F178" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="G178" s="4" t="n">
+        <v>1627</v>
+      </c>
+      <c r="H178" s="5" t="n">
+        <v>0.01623985009369144</v>
+      </c>
+      <c r="I178" s="5" t="n">
+        <v>0.01417939426510724</v>
+      </c>
+      <c r="J178" s="5" t="n">
+        <v>0.002060455828584207</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E179" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F179" s="4" t="n">
+        <v>1601</v>
+      </c>
+      <c r="G179" s="4" t="n">
+        <v>1561</v>
+      </c>
+      <c r="H179" s="5" t="n">
+        <v>-0.0249843847595253</v>
+      </c>
+      <c r="I179" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J179" s="5" t="n">
+        <v>-0.03033070676721003</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
           <t>9757</t>
         </is>
       </c>
-      <c r="C161" s="3" t="inlineStr">
+      <c r="C180" s="3" t="inlineStr">
         <is>
           <t>船井総研ホールディングス</t>
         </is>
       </c>
-      <c r="D161" s="2" t="n">
+      <c r="D180" s="2" t="n">
         <v>46300</v>
       </c>
-      <c r="E161" s="3" t="n">
+      <c r="E180" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F161" s="4" t="n">
+      <c r="F180" s="4" t="n">
         <v>1165</v>
       </c>
-      <c r="G161" s="4" t="n">
+      <c r="G180" s="4" t="n">
         <v>1158</v>
       </c>
-      <c r="H161" s="5" t="n">
+      <c r="H180" s="5" t="n">
         <v>-0.006008583690987125</v>
       </c>
-      <c r="I161" s="5" t="n">
+      <c r="I180" s="5" t="n">
         <v>0.01417939426510724</v>
       </c>
-      <c r="J161" s="5" t="n">
+      <c r="J180" s="5" t="n">
         <v>-0.02018797795609436</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>9757</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>船井総研ホールディングス</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E181" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F181" s="4" t="n">
+        <v>1165</v>
+      </c>
+      <c r="G181" s="4" t="n">
+        <v>1185</v>
+      </c>
+      <c r="H181" s="5" t="n">
+        <v>0.01716738197424893</v>
+      </c>
+      <c r="I181" s="5" t="n">
+        <v>0.005346322007684735</v>
+      </c>
+      <c r="J181" s="5" t="n">
+        <v>0.01182105996656419</v>
       </c>
     </row>
   </sheetData>
@@ -9398,7 +10118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9410,6 +10130,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9458,6 +10179,11 @@
           <t>2026-10-05</t>
         </is>
       </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -9491,6 +10217,7 @@
       <c r="I2" s="4" t="n">
         <v>2125</v>
       </c>
+      <c r="J2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -9524,6 +10251,7 @@
       <c r="I3" s="4" t="n">
         <v>422</v>
       </c>
+      <c r="J3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -9557,6 +10285,7 @@
       <c r="I4" s="4" t="n">
         <v>3360</v>
       </c>
+      <c r="J4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -9590,6 +10319,7 @@
       <c r="I5" s="4" t="n">
         <v>2362</v>
       </c>
+      <c r="J5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -9623,6 +10353,7 @@
       <c r="I6" s="4" t="n">
         <v>1620.5</v>
       </c>
+      <c r="J6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -9656,6 +10387,7 @@
       <c r="I7" s="4" t="n">
         <v>4655</v>
       </c>
+      <c r="J7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -9689,6 +10421,7 @@
       <c r="I8" s="4" t="n">
         <v>2022</v>
       </c>
+      <c r="J8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -9722,6 +10455,7 @@
       <c r="I9" s="4" t="n">
         <v>2809</v>
       </c>
+      <c r="J9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -9755,6 +10489,7 @@
       <c r="I10" s="4" t="n">
         <v>2235</v>
       </c>
+      <c r="J10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -9788,6 +10523,7 @@
       <c r="I11" s="4" t="n">
         <v>7191</v>
       </c>
+      <c r="J11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -9821,6 +10557,7 @@
       <c r="I12" s="4" t="n">
         <v>3924</v>
       </c>
+      <c r="J12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -9854,6 +10591,7 @@
       <c r="I13" s="4" t="n">
         <v>2484</v>
       </c>
+      <c r="J13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -9887,6 +10625,7 @@
       <c r="I14" s="4" t="n">
         <v>1926</v>
       </c>
+      <c r="J14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -9920,6 +10659,7 @@
       <c r="I15" s="4" t="n">
         <v>2647.5</v>
       </c>
+      <c r="J15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -9953,6 +10693,7 @@
       <c r="I16" s="4" t="n">
         <v>660</v>
       </c>
+      <c r="J16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -9986,6 +10727,7 @@
       <c r="I17" s="4" t="n">
         <v>3045</v>
       </c>
+      <c r="J17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -10019,6 +10761,7 @@
       <c r="I18" s="4" t="n">
         <v>892</v>
       </c>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -10052,6 +10795,7 @@
       <c r="I19" s="4" t="n">
         <v>1490</v>
       </c>
+      <c r="J19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -10085,6 +10829,7 @@
       <c r="I20" s="4" t="n">
         <v>1210</v>
       </c>
+      <c r="J20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -10118,6 +10863,7 @@
       <c r="I21" s="4" t="n">
         <v>1627</v>
       </c>
+      <c r="J21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -10145,6 +10891,7 @@
       <c r="I22" s="4" t="n">
         <v>2125</v>
       </c>
+      <c r="J22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -10172,6 +10919,7 @@
       <c r="I23" s="4" t="n">
         <v>422</v>
       </c>
+      <c r="J23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -10199,6 +10947,7 @@
       <c r="I24" s="4" t="n">
         <v>3360</v>
       </c>
+      <c r="J24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -10226,6 +10975,7 @@
       <c r="I25" s="4" t="n">
         <v>2362</v>
       </c>
+      <c r="J25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -10253,6 +11003,7 @@
       <c r="I26" s="4" t="n">
         <v>1620.5</v>
       </c>
+      <c r="J26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -10280,6 +11031,7 @@
       <c r="I27" s="4" t="n">
         <v>4655</v>
       </c>
+      <c r="J27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -10307,6 +11059,7 @@
       <c r="I28" s="4" t="n">
         <v>2022</v>
       </c>
+      <c r="J28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -10334,6 +11087,7 @@
       <c r="I29" s="4" t="n">
         <v>2809</v>
       </c>
+      <c r="J29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -10361,6 +11115,7 @@
       <c r="I30" s="4" t="n">
         <v>2235</v>
       </c>
+      <c r="J30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -10388,6 +11143,7 @@
       <c r="I31" s="4" t="n">
         <v>7191</v>
       </c>
+      <c r="J31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -10415,6 +11171,7 @@
       <c r="I32" s="4" t="n">
         <v>2484</v>
       </c>
+      <c r="J32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -10442,6 +11199,7 @@
       <c r="I33" s="4" t="n">
         <v>1926</v>
       </c>
+      <c r="J33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -10469,6 +11227,7 @@
       <c r="I34" s="4" t="n">
         <v>2647.5</v>
       </c>
+      <c r="J34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -10496,6 +11255,7 @@
       <c r="I35" s="4" t="n">
         <v>660</v>
       </c>
+      <c r="J35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -10523,6 +11283,7 @@
       <c r="I36" s="4" t="n">
         <v>3045</v>
       </c>
+      <c r="J36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -10550,6 +11311,7 @@
       <c r="I37" s="4" t="n">
         <v>892</v>
       </c>
+      <c r="J37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -10577,6 +11339,7 @@
       <c r="I38" s="4" t="n">
         <v>1490</v>
       </c>
+      <c r="J38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -10604,6 +11367,7 @@
       <c r="I39" s="4" t="n">
         <v>1210</v>
       </c>
+      <c r="J39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -10631,6 +11395,7 @@
       <c r="I40" s="4" t="n">
         <v>1627</v>
       </c>
+      <c r="J40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -10658,6 +11423,7 @@
       <c r="I41" s="4" t="n">
         <v>1158</v>
       </c>
+      <c r="J41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -10683,6 +11449,9 @@
       <c r="I42" s="4" t="n">
         <v>950</v>
       </c>
+      <c r="J42" s="4" t="n">
+        <v>935</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -10708,6 +11477,9 @@
       <c r="I43" s="4" t="n">
         <v>3870</v>
       </c>
+      <c r="J43" s="4" t="n">
+        <v>3845</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -10733,6 +11505,9 @@
       <c r="I44" s="4" t="n">
         <v>2125</v>
       </c>
+      <c r="J44" s="4" t="n">
+        <v>2157</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -10758,6 +11533,9 @@
       <c r="I45" s="4" t="n">
         <v>422</v>
       </c>
+      <c r="J45" s="4" t="n">
+        <v>433</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -10783,6 +11561,9 @@
       <c r="I46" s="4" t="n">
         <v>3360</v>
       </c>
+      <c r="J46" s="4" t="n">
+        <v>3415</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -10808,6 +11589,9 @@
       <c r="I47" s="4" t="n">
         <v>2362</v>
       </c>
+      <c r="J47" s="4" t="n">
+        <v>2389</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -10833,6 +11617,9 @@
       <c r="I48" s="4" t="n">
         <v>1620.5</v>
       </c>
+      <c r="J48" s="4" t="n">
+        <v>1637</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -10858,6 +11645,9 @@
       <c r="I49" s="4" t="n">
         <v>4655</v>
       </c>
+      <c r="J49" s="4" t="n">
+        <v>4745</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -10883,6 +11673,9 @@
       <c r="I50" s="4" t="n">
         <v>2022</v>
       </c>
+      <c r="J50" s="4" t="n">
+        <v>2133</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -10908,6 +11701,9 @@
       <c r="I51" s="4" t="n">
         <v>2809</v>
       </c>
+      <c r="J51" s="4" t="n">
+        <v>2814</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -10933,6 +11729,9 @@
       <c r="I52" s="4" t="n">
         <v>2235</v>
       </c>
+      <c r="J52" s="4" t="n">
+        <v>2247.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -10958,6 +11757,9 @@
       <c r="I53" s="4" t="n">
         <v>2484</v>
       </c>
+      <c r="J53" s="4" t="n">
+        <v>2485</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -10983,6 +11785,9 @@
       <c r="I54" s="4" t="n">
         <v>3947</v>
       </c>
+      <c r="J54" s="4" t="n">
+        <v>3828</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -11008,6 +11813,9 @@
       <c r="I55" s="4" t="n">
         <v>660</v>
       </c>
+      <c r="J55" s="4" t="n">
+        <v>695</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -11033,6 +11841,9 @@
       <c r="I56" s="4" t="n">
         <v>3045</v>
       </c>
+      <c r="J56" s="4" t="n">
+        <v>2918</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -11058,6 +11869,9 @@
       <c r="I57" s="4" t="n">
         <v>1490</v>
       </c>
+      <c r="J57" s="4" t="n">
+        <v>1431</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -11083,6 +11897,9 @@
       <c r="I58" s="4" t="n">
         <v>1210</v>
       </c>
+      <c r="J58" s="4" t="n">
+        <v>1241</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -11108,6 +11925,9 @@
       <c r="I59" s="4" t="n">
         <v>12765</v>
       </c>
+      <c r="J59" s="4" t="n">
+        <v>12445</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -11133,6 +11953,9 @@
       <c r="I60" s="4" t="n">
         <v>1627</v>
       </c>
+      <c r="J60" s="4" t="n">
+        <v>1561</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -11158,6 +11981,9 @@
       <c r="I61" s="4" t="n">
         <v>1158</v>
       </c>
+      <c r="J61" s="4" t="n">
+        <v>1185</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -11181,6 +12007,7 @@
       <c r="G62" s="4" t="n"/>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
+      <c r="J62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -11204,6 +12031,7 @@
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
+      <c r="J63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -11227,6 +12055,7 @@
       <c r="G64" s="4" t="n"/>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
+      <c r="J64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -11250,6 +12079,7 @@
       <c r="G65" s="4" t="n"/>
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
+      <c r="J65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -11273,6 +12103,7 @@
       <c r="G66" s="4" t="n"/>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
+      <c r="J66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -11296,6 +12127,7 @@
       <c r="G67" s="4" t="n"/>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
+      <c r="J67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -11319,6 +12151,7 @@
       <c r="G68" s="4" t="n"/>
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
+      <c r="J68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -11342,6 +12175,7 @@
       <c r="G69" s="4" t="n"/>
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
+      <c r="J69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -11365,6 +12199,7 @@
       <c r="G70" s="4" t="n"/>
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
+      <c r="J70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -11388,6 +12223,7 @@
       <c r="G71" s="4" t="n"/>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
+      <c r="J71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -11411,6 +12247,7 @@
       <c r="G72" s="4" t="n"/>
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
+      <c r="J72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -11434,6 +12271,7 @@
       <c r="G73" s="4" t="n"/>
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="n"/>
+      <c r="J73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -11457,6 +12295,7 @@
       <c r="G74" s="4" t="n"/>
       <c r="H74" s="4" t="n"/>
       <c r="I74" s="4" t="n"/>
+      <c r="J74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -11480,6 +12319,7 @@
       <c r="G75" s="4" t="n"/>
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
+      <c r="J75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -11503,6 +12343,7 @@
       <c r="G76" s="4" t="n"/>
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
+      <c r="J76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -11526,6 +12367,7 @@
       <c r="G77" s="4" t="n"/>
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -11549,6 +12391,7 @@
       <c r="G78" s="4" t="n"/>
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
+      <c r="J78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -11572,6 +12415,7 @@
       <c r="G79" s="4" t="n"/>
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
+      <c r="J79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -11595,6 +12439,7 @@
       <c r="G80" s="4" t="n"/>
       <c r="H80" s="4" t="n"/>
       <c r="I80" s="4" t="n"/>
+      <c r="J80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -11618,6 +12463,7 @@
       <c r="G81" s="4" t="n"/>
       <c r="H81" s="4" t="n"/>
       <c r="I81" s="4" t="n"/>
+      <c r="J81" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record entry prices 2026-10-17
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="週次ピック" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="価格推移ログ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="価格推移(ピボット)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="週次ピック" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="価格推移ログ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="価格推移(ピボット)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3547,6 +3547,766 @@
       </c>
       <c r="J81" s="4" t="n">
         <v>432.5</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>証券、商品先物取引業</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="G82" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="I82" s="4" t="n">
+        <v>1572</v>
+      </c>
+      <c r="J82" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="G83" s="3" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="H83" s="3" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="I83" s="4" t="n">
+        <v>2786</v>
+      </c>
+      <c r="J83" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>電気・ガス業</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="I84" s="4" t="n">
+        <v>2378</v>
+      </c>
+      <c r="J84" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>食料品</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="I85" s="4" t="n">
+        <v>2180</v>
+      </c>
+      <c r="J85" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="I86" s="4" t="n">
+        <v>1682</v>
+      </c>
+      <c r="J86" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="I87" s="4" t="n">
+        <v>703</v>
+      </c>
+      <c r="J87" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>医薬品</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="I88" s="4" t="n">
+        <v>2418.5</v>
+      </c>
+      <c r="J88" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="I89" s="4" t="n">
+        <v>3679</v>
+      </c>
+      <c r="J89" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>97.3</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>1162</v>
+      </c>
+      <c r="J90" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>輸送用機器</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="G91" s="3" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="I91" s="4" t="n">
+        <v>1430</v>
+      </c>
+      <c r="J91" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="G92" s="3" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="I92" s="4" t="n">
+        <v>2717</v>
+      </c>
+      <c r="J92" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G93" s="3" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="H93" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="I93" s="4" t="n">
+        <v>4820</v>
+      </c>
+      <c r="J93" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="G94" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I94" s="4" t="n">
+        <v>458</v>
+      </c>
+      <c r="J94" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="G95" s="3" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="H95" s="3" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="I95" s="4" t="n">
+        <v>1324</v>
+      </c>
+      <c r="J95" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="G96" s="3" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="I96" s="4" t="n">
+        <v>3860</v>
+      </c>
+      <c r="J96" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="G97" s="3" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="H97" s="3" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="I97" s="4" t="n">
+        <v>854</v>
+      </c>
+      <c r="J97" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G98" s="3" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="H98" s="3" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="I98" s="4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J98" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F99" s="3" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="G99" s="3" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="H99" s="3" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="I99" s="4" t="n">
+        <v>2227</v>
+      </c>
+      <c r="J99" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G100" s="3" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H100" s="3" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="I100" s="4" t="n">
+        <v>2613</v>
+      </c>
+      <c r="J100" s="4" t="n">
+        <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>1879</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>新日本建設</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="G101" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="H101" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="I101" s="4" t="n">
+        <v>2197</v>
+      </c>
+      <c r="J101" s="4" t="n">
+        <v>428.3999938964844</v>
       </c>
     </row>
   </sheetData>
@@ -10118,7 +10878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12465,6 +13225,486 @@
       <c r="I81" s="4" t="n"/>
       <c r="J81" s="4" t="n"/>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>1879</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>新日本建設</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="n">
+        <v>2197</v>
+      </c>
+      <c r="E82" s="4" t="n"/>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
+      <c r="J82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="n">
+        <v>3860</v>
+      </c>
+      <c r="E83" s="4" t="n"/>
+      <c r="F83" s="4" t="n"/>
+      <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
+      <c r="J83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="n">
+        <v>2180</v>
+      </c>
+      <c r="E84" s="4" t="n"/>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
+      <c r="J84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="n">
+        <v>458</v>
+      </c>
+      <c r="E85" s="4" t="n"/>
+      <c r="F85" s="4" t="n"/>
+      <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
+      <c r="J85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="n">
+        <v>2378</v>
+      </c>
+      <c r="E86" s="4" t="n"/>
+      <c r="F86" s="4" t="n"/>
+      <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
+      <c r="I86" s="4" t="n"/>
+      <c r="J86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="n">
+        <v>1682</v>
+      </c>
+      <c r="E87" s="4" t="n"/>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
+      <c r="J87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="n">
+        <v>4820</v>
+      </c>
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="n">
+        <v>2227</v>
+      </c>
+      <c r="E89" s="4" t="n"/>
+      <c r="F89" s="4" t="n"/>
+      <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
+      <c r="J89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="n">
+        <v>1162</v>
+      </c>
+      <c r="E90" s="4" t="n"/>
+      <c r="F90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n"/>
+      <c r="I90" s="4" t="n"/>
+      <c r="J90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="n">
+        <v>2717</v>
+      </c>
+      <c r="E91" s="4" t="n"/>
+      <c r="F91" s="4" t="n"/>
+      <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
+      <c r="I91" s="4" t="n"/>
+      <c r="J91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="n">
+        <v>2418.5</v>
+      </c>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="n">
+        <v>2613</v>
+      </c>
+      <c r="E93" s="4" t="n"/>
+      <c r="F93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" s="4" t="n"/>
+      <c r="J93" s="4" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="n">
+        <v>3679</v>
+      </c>
+      <c r="E94" s="4" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
+      <c r="J94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="n">
+        <v>703</v>
+      </c>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="4" t="n"/>
+      <c r="J95" s="4" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="n">
+        <v>2786</v>
+      </c>
+      <c r="E96" s="4" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
+      <c r="J96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>854</v>
+      </c>
+      <c r="E97" s="4" t="n"/>
+      <c r="F97" s="4" t="n"/>
+      <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
+      <c r="I97" s="4" t="n"/>
+      <c r="J97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E98" s="4" t="n"/>
+      <c r="F98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
+      <c r="I98" s="4" t="n"/>
+      <c r="J98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="n">
+        <v>1430</v>
+      </c>
+      <c r="E99" s="4" t="n"/>
+      <c r="F99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="n">
+        <v>1324</v>
+      </c>
+      <c r="E100" s="4" t="n"/>
+      <c r="F100" s="4" t="n"/>
+      <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n"/>
+      <c r="I100" s="4" t="n"/>
+      <c r="J100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="n">
+        <v>1572</v>
+      </c>
+      <c r="E101" s="4" t="n"/>
+      <c r="F101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Performance check 2026-10-10 -> 2026-10-17
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -4320,7 +4320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10867,6 +10867,726 @@
         <v>0.01182105996656419</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E182" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F182" s="4" t="n">
+        <v>3845</v>
+      </c>
+      <c r="G182" s="4" t="n">
+        <v>3860</v>
+      </c>
+      <c r="H182" s="5" t="n">
+        <v>0.003901170351105332</v>
+      </c>
+      <c r="I182" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J182" s="5" t="n">
+        <v>0.01338095324940736</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E183" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F183" s="4" t="n">
+        <v>2157</v>
+      </c>
+      <c r="G183" s="4" t="n">
+        <v>2180</v>
+      </c>
+      <c r="H183" s="5" t="n">
+        <v>0.01066295781177561</v>
+      </c>
+      <c r="I183" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J183" s="5" t="n">
+        <v>0.02014274071007764</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E184" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F184" s="4" t="n">
+        <v>433</v>
+      </c>
+      <c r="G184" s="4" t="n">
+        <v>458</v>
+      </c>
+      <c r="H184" s="5" t="n">
+        <v>0.05773672055427252</v>
+      </c>
+      <c r="I184" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J184" s="5" t="n">
+        <v>0.06721650345257454</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>3110</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>日東紡績</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E185" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F185" s="4" t="n">
+        <v>3415</v>
+      </c>
+      <c r="G185" s="4" t="n">
+        <v>2989</v>
+      </c>
+      <c r="H185" s="5" t="n">
+        <v>-0.1247437774524158</v>
+      </c>
+      <c r="I185" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J185" s="5" t="n">
+        <v>-0.1152639945541138</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E186" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F186" s="4" t="n">
+        <v>2389</v>
+      </c>
+      <c r="G186" s="4" t="n">
+        <v>2378</v>
+      </c>
+      <c r="H186" s="5" t="n">
+        <v>-0.004604437002930097</v>
+      </c>
+      <c r="I186" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J186" s="5" t="n">
+        <v>0.004875345895371927</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E187" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F187" s="4" t="n">
+        <v>1637</v>
+      </c>
+      <c r="G187" s="4" t="n">
+        <v>1682</v>
+      </c>
+      <c r="H187" s="5" t="n">
+        <v>0.02748930971288943</v>
+      </c>
+      <c r="I187" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J187" s="5" t="n">
+        <v>0.03696909261119145</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E188" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F188" s="4" t="n">
+        <v>4745</v>
+      </c>
+      <c r="G188" s="4" t="n">
+        <v>4820</v>
+      </c>
+      <c r="H188" s="5" t="n">
+        <v>0.01580611169652266</v>
+      </c>
+      <c r="I188" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J188" s="5" t="n">
+        <v>0.02528589459482468</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E189" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F189" s="4" t="n">
+        <v>2133</v>
+      </c>
+      <c r="G189" s="4" t="n">
+        <v>2227</v>
+      </c>
+      <c r="H189" s="5" t="n">
+        <v>0.04406938584153774</v>
+      </c>
+      <c r="I189" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J189" s="5" t="n">
+        <v>0.05354916873983976</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E190" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F190" s="4" t="n">
+        <v>1134</v>
+      </c>
+      <c r="G190" s="4" t="n">
+        <v>1162</v>
+      </c>
+      <c r="H190" s="5" t="n">
+        <v>0.02469135802469136</v>
+      </c>
+      <c r="I190" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J190" s="5" t="n">
+        <v>0.03417114092299338</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>3932</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>アカツキ</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E191" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F191" s="4" t="n">
+        <v>1295</v>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>1382</v>
+      </c>
+      <c r="H191" s="5" t="n">
+        <v>0.06718146718146718</v>
+      </c>
+      <c r="I191" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J191" s="5" t="n">
+        <v>0.07666125007976921</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E192" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F192" s="4" t="n">
+        <v>2814</v>
+      </c>
+      <c r="G192" s="4" t="n">
+        <v>2717</v>
+      </c>
+      <c r="H192" s="5" t="n">
+        <v>-0.03447050461975835</v>
+      </c>
+      <c r="I192" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J192" s="5" t="n">
+        <v>-0.02499072172145633</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E193" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F193" s="4" t="n">
+        <v>2247.5</v>
+      </c>
+      <c r="G193" s="4" t="n">
+        <v>2418.5</v>
+      </c>
+      <c r="H193" s="5" t="n">
+        <v>0.0760845383759733</v>
+      </c>
+      <c r="I193" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J193" s="5" t="n">
+        <v>0.08556432127427532</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E194" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F194" s="4" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G194" s="4" t="n">
+        <v>2613</v>
+      </c>
+      <c r="H194" s="5" t="n">
+        <v>0.05150905432595573</v>
+      </c>
+      <c r="I194" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J194" s="5" t="n">
+        <v>0.06098883722425776</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E195" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F195" s="4" t="n">
+        <v>3828</v>
+      </c>
+      <c r="G195" s="4" t="n">
+        <v>3679</v>
+      </c>
+      <c r="H195" s="5" t="n">
+        <v>-0.03892371995820271</v>
+      </c>
+      <c r="I195" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J195" s="5" t="n">
+        <v>-0.02944393705990069</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E196" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F196" s="4" t="n">
+        <v>695</v>
+      </c>
+      <c r="G196" s="4" t="n">
+        <v>703</v>
+      </c>
+      <c r="H196" s="5" t="n">
+        <v>0.01151079136690648</v>
+      </c>
+      <c r="I196" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J196" s="5" t="n">
+        <v>0.0209905742652085</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E197" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>2918</v>
+      </c>
+      <c r="G197" s="4" t="n">
+        <v>2786</v>
+      </c>
+      <c r="H197" s="5" t="n">
+        <v>-0.04523646333104867</v>
+      </c>
+      <c r="I197" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J197" s="5" t="n">
+        <v>-0.03575668043274664</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E198" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F198" s="4" t="n">
+        <v>1978</v>
+      </c>
+      <c r="G198" s="4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="H198" s="5" t="n">
+        <v>0.019211324570273</v>
+      </c>
+      <c r="I198" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J198" s="5" t="n">
+        <v>0.02869110746857503</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E199" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F199" s="4" t="n">
+        <v>1431</v>
+      </c>
+      <c r="G199" s="4" t="n">
+        <v>1430</v>
+      </c>
+      <c r="H199" s="5" t="n">
+        <v>-0.0006988120195667365</v>
+      </c>
+      <c r="I199" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J199" s="5" t="n">
+        <v>0.008780970878735287</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E200" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F200" s="4" t="n">
+        <v>1241</v>
+      </c>
+      <c r="G200" s="4" t="n">
+        <v>1324</v>
+      </c>
+      <c r="H200" s="5" t="n">
+        <v>0.06688154713940371</v>
+      </c>
+      <c r="I200" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J200" s="5" t="n">
+        <v>0.07636133003770573</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E201" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F201" s="4" t="n">
+        <v>1561</v>
+      </c>
+      <c r="G201" s="4" t="n">
+        <v>1572</v>
+      </c>
+      <c r="H201" s="5" t="n">
+        <v>0.007046764894298526</v>
+      </c>
+      <c r="I201" s="5" t="n">
+        <v>-0.009479782898302024</v>
+      </c>
+      <c r="J201" s="5" t="n">
+        <v>0.01652654779260055</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10878,7 +11598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10891,6 +11611,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10944,6 +11665,11 @@
           <t>2026-10-10</t>
         </is>
       </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -10978,6 +11704,7 @@
         <v>2125</v>
       </c>
       <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -11012,6 +11739,7 @@
         <v>422</v>
       </c>
       <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -11046,6 +11774,7 @@
         <v>3360</v>
       </c>
       <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -11080,6 +11809,7 @@
         <v>2362</v>
       </c>
       <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -11114,6 +11844,7 @@
         <v>1620.5</v>
       </c>
       <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -11148,6 +11879,7 @@
         <v>4655</v>
       </c>
       <c r="J7" s="4" t="n"/>
+      <c r="K7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -11182,6 +11914,7 @@
         <v>2022</v>
       </c>
       <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -11216,6 +11949,7 @@
         <v>2809</v>
       </c>
       <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -11250,6 +11984,7 @@
         <v>2235</v>
       </c>
       <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -11284,6 +12019,7 @@
         <v>7191</v>
       </c>
       <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -11318,6 +12054,7 @@
         <v>3924</v>
       </c>
       <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -11352,6 +12089,7 @@
         <v>2484</v>
       </c>
       <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -11386,6 +12124,7 @@
         <v>1926</v>
       </c>
       <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -11420,6 +12159,7 @@
         <v>2647.5</v>
       </c>
       <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -11454,6 +12194,7 @@
         <v>660</v>
       </c>
       <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -11488,6 +12229,7 @@
         <v>3045</v>
       </c>
       <c r="J17" s="4" t="n"/>
+      <c r="K17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -11522,6 +12264,7 @@
         <v>892</v>
       </c>
       <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -11556,6 +12299,7 @@
         <v>1490</v>
       </c>
       <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -11590,6 +12334,7 @@
         <v>1210</v>
       </c>
       <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -11624,6 +12369,7 @@
         <v>1627</v>
       </c>
       <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -11652,6 +12398,7 @@
         <v>2125</v>
       </c>
       <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -11680,6 +12427,7 @@
         <v>422</v>
       </c>
       <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -11708,6 +12456,7 @@
         <v>3360</v>
       </c>
       <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -11736,6 +12485,7 @@
         <v>2362</v>
       </c>
       <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -11764,6 +12514,7 @@
         <v>1620.5</v>
       </c>
       <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -11792,6 +12543,7 @@
         <v>4655</v>
       </c>
       <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -11820,6 +12572,7 @@
         <v>2022</v>
       </c>
       <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -11848,6 +12601,7 @@
         <v>2809</v>
       </c>
       <c r="J29" s="4" t="n"/>
+      <c r="K29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -11876,6 +12630,7 @@
         <v>2235</v>
       </c>
       <c r="J30" s="4" t="n"/>
+      <c r="K30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -11904,6 +12659,7 @@
         <v>7191</v>
       </c>
       <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -11932,6 +12688,7 @@
         <v>2484</v>
       </c>
       <c r="J32" s="4" t="n"/>
+      <c r="K32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -11960,6 +12717,7 @@
         <v>1926</v>
       </c>
       <c r="J33" s="4" t="n"/>
+      <c r="K33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -11988,6 +12746,7 @@
         <v>2647.5</v>
       </c>
       <c r="J34" s="4" t="n"/>
+      <c r="K34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -12016,6 +12775,7 @@
         <v>660</v>
       </c>
       <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -12044,6 +12804,7 @@
         <v>3045</v>
       </c>
       <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -12072,6 +12833,7 @@
         <v>892</v>
       </c>
       <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -12100,6 +12862,7 @@
         <v>1490</v>
       </c>
       <c r="J38" s="4" t="n"/>
+      <c r="K38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -12128,6 +12891,7 @@
         <v>1210</v>
       </c>
       <c r="J39" s="4" t="n"/>
+      <c r="K39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -12156,6 +12920,7 @@
         <v>1627</v>
       </c>
       <c r="J40" s="4" t="n"/>
+      <c r="K40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -12184,6 +12949,7 @@
         <v>1158</v>
       </c>
       <c r="J41" s="4" t="n"/>
+      <c r="K41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -12212,6 +12978,7 @@
       <c r="J42" s="4" t="n">
         <v>935</v>
       </c>
+      <c r="K42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -12240,6 +13007,7 @@
       <c r="J43" s="4" t="n">
         <v>3845</v>
       </c>
+      <c r="K43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -12268,6 +13036,7 @@
       <c r="J44" s="4" t="n">
         <v>2157</v>
       </c>
+      <c r="K44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -12296,6 +13065,7 @@
       <c r="J45" s="4" t="n">
         <v>433</v>
       </c>
+      <c r="K45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -12324,6 +13094,7 @@
       <c r="J46" s="4" t="n">
         <v>3415</v>
       </c>
+      <c r="K46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -12352,6 +13123,7 @@
       <c r="J47" s="4" t="n">
         <v>2389</v>
       </c>
+      <c r="K47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -12380,6 +13152,7 @@
       <c r="J48" s="4" t="n">
         <v>1637</v>
       </c>
+      <c r="K48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -12408,6 +13181,7 @@
       <c r="J49" s="4" t="n">
         <v>4745</v>
       </c>
+      <c r="K49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -12436,6 +13210,7 @@
       <c r="J50" s="4" t="n">
         <v>2133</v>
       </c>
+      <c r="K50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -12464,6 +13239,7 @@
       <c r="J51" s="4" t="n">
         <v>2814</v>
       </c>
+      <c r="K51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -12492,6 +13268,7 @@
       <c r="J52" s="4" t="n">
         <v>2247.5</v>
       </c>
+      <c r="K52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -12520,6 +13297,7 @@
       <c r="J53" s="4" t="n">
         <v>2485</v>
       </c>
+      <c r="K53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -12548,6 +13326,7 @@
       <c r="J54" s="4" t="n">
         <v>3828</v>
       </c>
+      <c r="K54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -12576,6 +13355,7 @@
       <c r="J55" s="4" t="n">
         <v>695</v>
       </c>
+      <c r="K55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -12604,6 +13384,7 @@
       <c r="J56" s="4" t="n">
         <v>2918</v>
       </c>
+      <c r="K56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -12632,6 +13413,7 @@
       <c r="J57" s="4" t="n">
         <v>1431</v>
       </c>
+      <c r="K57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -12660,6 +13442,7 @@
       <c r="J58" s="4" t="n">
         <v>1241</v>
       </c>
+      <c r="K58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -12688,6 +13471,7 @@
       <c r="J59" s="4" t="n">
         <v>12445</v>
       </c>
+      <c r="K59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -12716,6 +13500,7 @@
       <c r="J60" s="4" t="n">
         <v>1561</v>
       </c>
+      <c r="K60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -12744,6 +13529,7 @@
       <c r="J61" s="4" t="n">
         <v>1185</v>
       </c>
+      <c r="K61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -12768,6 +13554,9 @@
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="4" t="n"/>
+      <c r="K62" s="4" t="n">
+        <v>3860</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -12792,6 +13581,9 @@
       <c r="H63" s="4" t="n"/>
       <c r="I63" s="4" t="n"/>
       <c r="J63" s="4" t="n"/>
+      <c r="K63" s="4" t="n">
+        <v>2180</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -12816,6 +13608,9 @@
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
       <c r="J64" s="4" t="n"/>
+      <c r="K64" s="4" t="n">
+        <v>458</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -12840,6 +13635,9 @@
       <c r="H65" s="4" t="n"/>
       <c r="I65" s="4" t="n"/>
       <c r="J65" s="4" t="n"/>
+      <c r="K65" s="4" t="n">
+        <v>2989</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -12864,6 +13662,9 @@
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
       <c r="J66" s="4" t="n"/>
+      <c r="K66" s="4" t="n">
+        <v>2378</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -12888,6 +13689,9 @@
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
       <c r="J67" s="4" t="n"/>
+      <c r="K67" s="4" t="n">
+        <v>1682</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -12912,6 +13716,9 @@
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
       <c r="J68" s="4" t="n"/>
+      <c r="K68" s="4" t="n">
+        <v>4820</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -12936,6 +13743,9 @@
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
       <c r="J69" s="4" t="n"/>
+      <c r="K69" s="4" t="n">
+        <v>2227</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -12960,6 +13770,9 @@
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="n">
+        <v>1162</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -12984,6 +13797,9 @@
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
       <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="n">
+        <v>1382</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -13008,6 +13824,9 @@
       <c r="H72" s="4" t="n"/>
       <c r="I72" s="4" t="n"/>
       <c r="J72" s="4" t="n"/>
+      <c r="K72" s="4" t="n">
+        <v>2717</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -13032,6 +13851,9 @@
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="n"/>
       <c r="J73" s="4" t="n"/>
+      <c r="K73" s="4" t="n">
+        <v>2418.5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -13056,6 +13878,9 @@
       <c r="H74" s="4" t="n"/>
       <c r="I74" s="4" t="n"/>
       <c r="J74" s="4" t="n"/>
+      <c r="K74" s="4" t="n">
+        <v>2613</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -13080,6 +13905,9 @@
       <c r="H75" s="4" t="n"/>
       <c r="I75" s="4" t="n"/>
       <c r="J75" s="4" t="n"/>
+      <c r="K75" s="4" t="n">
+        <v>3679</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -13104,6 +13932,9 @@
       <c r="H76" s="4" t="n"/>
       <c r="I76" s="4" t="n"/>
       <c r="J76" s="4" t="n"/>
+      <c r="K76" s="4" t="n">
+        <v>703</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -13128,6 +13959,9 @@
       <c r="H77" s="4" t="n"/>
       <c r="I77" s="4" t="n"/>
       <c r="J77" s="4" t="n"/>
+      <c r="K77" s="4" t="n">
+        <v>2786</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -13152,6 +13986,9 @@
       <c r="H78" s="4" t="n"/>
       <c r="I78" s="4" t="n"/>
       <c r="J78" s="4" t="n"/>
+      <c r="K78" s="4" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -13176,6 +14013,9 @@
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
       <c r="J79" s="4" t="n"/>
+      <c r="K79" s="4" t="n">
+        <v>1430</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -13200,6 +14040,9 @@
       <c r="H80" s="4" t="n"/>
       <c r="I80" s="4" t="n"/>
       <c r="J80" s="4" t="n"/>
+      <c r="K80" s="4" t="n">
+        <v>1324</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -13224,6 +14067,9 @@
       <c r="H81" s="4" t="n"/>
       <c r="I81" s="4" t="n"/>
       <c r="J81" s="4" t="n"/>
+      <c r="K81" s="4" t="n">
+        <v>1572</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -13248,6 +14094,7 @@
       <c r="H82" s="4" t="n"/>
       <c r="I82" s="4" t="n"/>
       <c r="J82" s="4" t="n"/>
+      <c r="K82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -13272,6 +14119,7 @@
       <c r="H83" s="4" t="n"/>
       <c r="I83" s="4" t="n"/>
       <c r="J83" s="4" t="n"/>
+      <c r="K83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -13296,6 +14144,7 @@
       <c r="H84" s="4" t="n"/>
       <c r="I84" s="4" t="n"/>
       <c r="J84" s="4" t="n"/>
+      <c r="K84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -13320,6 +14169,7 @@
       <c r="H85" s="4" t="n"/>
       <c r="I85" s="4" t="n"/>
       <c r="J85" s="4" t="n"/>
+      <c r="K85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -13344,6 +14194,7 @@
       <c r="H86" s="4" t="n"/>
       <c r="I86" s="4" t="n"/>
       <c r="J86" s="4" t="n"/>
+      <c r="K86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -13368,6 +14219,7 @@
       <c r="H87" s="4" t="n"/>
       <c r="I87" s="4" t="n"/>
       <c r="J87" s="4" t="n"/>
+      <c r="K87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -13392,6 +14244,7 @@
       <c r="H88" s="4" t="n"/>
       <c r="I88" s="4" t="n"/>
       <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -13416,6 +14269,7 @@
       <c r="H89" s="4" t="n"/>
       <c r="I89" s="4" t="n"/>
       <c r="J89" s="4" t="n"/>
+      <c r="K89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -13440,6 +14294,7 @@
       <c r="H90" s="4" t="n"/>
       <c r="I90" s="4" t="n"/>
       <c r="J90" s="4" t="n"/>
+      <c r="K90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -13464,6 +14319,7 @@
       <c r="H91" s="4" t="n"/>
       <c r="I91" s="4" t="n"/>
       <c r="J91" s="4" t="n"/>
+      <c r="K91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -13488,6 +14344,7 @@
       <c r="H92" s="4" t="n"/>
       <c r="I92" s="4" t="n"/>
       <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -13512,6 +14369,7 @@
       <c r="H93" s="4" t="n"/>
       <c r="I93" s="4" t="n"/>
       <c r="J93" s="4" t="n"/>
+      <c r="K93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -13536,6 +14394,7 @@
       <c r="H94" s="4" t="n"/>
       <c r="I94" s="4" t="n"/>
       <c r="J94" s="4" t="n"/>
+      <c r="K94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -13560,6 +14419,7 @@
       <c r="H95" s="4" t="n"/>
       <c r="I95" s="4" t="n"/>
       <c r="J95" s="4" t="n"/>
+      <c r="K95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -13584,6 +14444,7 @@
       <c r="H96" s="4" t="n"/>
       <c r="I96" s="4" t="n"/>
       <c r="J96" s="4" t="n"/>
+      <c r="K96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -13608,6 +14469,7 @@
       <c r="H97" s="4" t="n"/>
       <c r="I97" s="4" t="n"/>
       <c r="J97" s="4" t="n"/>
+      <c r="K97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -13632,6 +14494,7 @@
       <c r="H98" s="4" t="n"/>
       <c r="I98" s="4" t="n"/>
       <c r="J98" s="4" t="n"/>
+      <c r="K98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -13656,6 +14519,7 @@
       <c r="H99" s="4" t="n"/>
       <c r="I99" s="4" t="n"/>
       <c r="J99" s="4" t="n"/>
+      <c r="K99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -13680,6 +14544,7 @@
       <c r="H100" s="4" t="n"/>
       <c r="I100" s="4" t="n"/>
       <c r="J100" s="4" t="n"/>
+      <c r="K100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -13704,6 +14569,7 @@
       <c r="H101" s="4" t="n"/>
       <c r="I101" s="4" t="n"/>
       <c r="J101" s="4" t="n"/>
+      <c r="K101" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Record entry prices 2026-10-24
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -454,7 +454,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2064,7 +2064,7 @@
         <v>1601</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="43">
@@ -2102,7 +2102,7 @@
         <v>2345</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="44">
@@ -2140,7 +2140,7 @@
         <v>3370</v>
       </c>
       <c r="J44" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="45">
@@ -2178,7 +2178,7 @@
         <v>952</v>
       </c>
       <c r="J45" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="46">
@@ -2216,7 +2216,7 @@
         <v>3050</v>
       </c>
       <c r="J46" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="47">
@@ -2254,7 +2254,7 @@
         <v>670</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="48">
@@ -2292,7 +2292,7 @@
         <v>3758</v>
       </c>
       <c r="J48" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="49">
@@ -2330,7 +2330,7 @@
         <v>2119</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="50">
@@ -2368,7 +2368,7 @@
         <v>1466</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="51">
@@ -2406,7 +2406,7 @@
         <v>1645.5</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="52">
@@ -2444,7 +2444,7 @@
         <v>12100</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="53">
@@ -2482,7 +2482,7 @@
         <v>424</v>
       </c>
       <c r="J53" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="54">
@@ -2520,7 +2520,7 @@
         <v>2245</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="55">
@@ -2558,7 +2558,7 @@
         <v>2791</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="56">
@@ -2596,7 +2596,7 @@
         <v>2038</v>
       </c>
       <c r="J56" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="57">
@@ -2634,7 +2634,7 @@
         <v>1209</v>
       </c>
       <c r="J57" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="58">
@@ -2672,7 +2672,7 @@
         <v>2450</v>
       </c>
       <c r="J58" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="59">
@@ -2710,7 +2710,7 @@
         <v>4710</v>
       </c>
       <c r="J59" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="60">
@@ -2748,7 +2748,7 @@
         <v>3835</v>
       </c>
       <c r="J60" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="61">
@@ -2786,7 +2786,7 @@
         <v>1165</v>
       </c>
       <c r="J61" s="4" t="n">
-        <v>430.2000122070313</v>
+        <v>430.2000122070312</v>
       </c>
     </row>
     <row r="62">
@@ -4307,6 +4307,766 @@
       </c>
       <c r="J101" s="4" t="n">
         <v>428.3999938964844</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="I102" s="4" t="n">
+        <v>2704</v>
+      </c>
+      <c r="J102" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>電気・ガス業</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="H103" s="3" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="I103" s="4" t="n">
+        <v>2350</v>
+      </c>
+      <c r="J103" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>食料品</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="G104" s="3" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="H104" s="3" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="I104" s="4" t="n">
+        <v>2205</v>
+      </c>
+      <c r="J104" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>ガラス・土石製品</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="G105" s="3" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="H105" s="3" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="I105" s="4" t="n">
+        <v>3389</v>
+      </c>
+      <c r="J105" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>サービス業</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G106" s="3" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="I106" s="4" t="n">
+        <v>702</v>
+      </c>
+      <c r="J106" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="H107" s="3" t="n">
+        <v>97.2</v>
+      </c>
+      <c r="I107" s="4" t="n">
+        <v>1112.5</v>
+      </c>
+      <c r="J107" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>輸送用機器</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="G108" s="3" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="I108" s="4" t="n">
+        <v>1361</v>
+      </c>
+      <c r="J108" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G109" s="3" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="H109" s="3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="I109" s="4" t="n">
+        <v>1658</v>
+      </c>
+      <c r="J109" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>医薬品</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G110" s="3" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>2512</v>
+      </c>
+      <c r="J110" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="G111" s="3" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="I111" s="4" t="n">
+        <v>2585</v>
+      </c>
+      <c r="J111" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>8739</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>スパークス・グループ</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>証券、商品先物取引業</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="G112" s="3" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="I112" s="4" t="n">
+        <v>2438</v>
+      </c>
+      <c r="J112" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="G113" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="H113" s="3" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="I113" s="4" t="n">
+        <v>4860</v>
+      </c>
+      <c r="J113" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="G114" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="I114" s="4" t="n">
+        <v>3695</v>
+      </c>
+      <c r="J114" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="G115" s="3" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="H115" s="3" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="I115" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="J115" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>4187</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>大阪有機化学工業</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>化学</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F116" s="3" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="G116" s="3" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="I116" s="4" t="n">
+        <v>4340</v>
+      </c>
+      <c r="J116" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>情報・通信業</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="F117" s="3" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="G117" s="3" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="H117" s="3" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="I117" s="4" t="n">
+        <v>452</v>
+      </c>
+      <c r="J117" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>ゴム製品</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="G118" s="3" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="I118" s="4" t="n">
+        <v>2582</v>
+      </c>
+      <c r="J118" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F119" s="3" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="G119" s="3" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="H119" s="3" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="I119" s="4" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J119" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>電気機器</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F120" s="3" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="G120" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="I120" s="4" t="n">
+        <v>857</v>
+      </c>
+      <c r="J120" s="4" t="n">
+        <v>416.2999877929688</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>1879</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>新日本建設</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>建設業</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F121" s="3" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="G121" s="3" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="H121" s="3" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="I121" s="4" t="n">
+        <v>2178</v>
+      </c>
+      <c r="J121" s="4" t="n">
+        <v>416.2999877929688</v>
       </c>
     </row>
   </sheetData>
@@ -8017,7 +8777,7 @@
         <v>-0.07305336832895888</v>
       </c>
       <c r="I102" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J102" s="5" t="n">
         <v>-0.07282102905688422</v>
@@ -8089,7 +8849,7 @@
         <v>-0.02752293577981652</v>
       </c>
       <c r="I104" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J104" s="5" t="n">
         <v>-0.02729059650774185</v>
@@ -8161,7 +8921,7 @@
         <v>0.1308724832214765</v>
       </c>
       <c r="I106" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J106" s="5" t="n">
         <v>0.1311048224935512</v>
@@ -8233,7 +8993,7 @@
         <v>-0.03735632183908046</v>
       </c>
       <c r="I108" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J108" s="5" t="n">
         <v>-0.0371239825670058</v>
@@ -8305,7 +9065,7 @@
         <v>-0.01526032315978456</v>
       </c>
       <c r="I110" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J110" s="5" t="n">
         <v>-0.01502798388770989</v>
@@ -8377,7 +9137,7 @@
         <v>-0.02986611740473738</v>
       </c>
       <c r="I112" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J112" s="5" t="n">
         <v>-0.02963377813266272</v>
@@ -8449,7 +9209,7 @@
         <v>-0.05297397769516728</v>
       </c>
       <c r="I114" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J114" s="5" t="n">
         <v>-0.05274163842309262</v>
@@ -8521,7 +9281,7 @@
         <v>-0.03692201518288475</v>
       </c>
       <c r="I116" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J116" s="5" t="n">
         <v>-0.03668967591081009</v>
@@ -8593,7 +9353,7 @@
         <v>-0.06419341392246769</v>
       </c>
       <c r="I118" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J118" s="5" t="n">
         <v>-0.06396107465039302</v>
@@ -8665,7 +9425,7 @@
         <v>0.0107357572287432</v>
       </c>
       <c r="I120" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J120" s="5" t="n">
         <v>0.01096809650081787</v>
@@ -8737,7 +9497,7 @@
         <v>-0.03047091412742382</v>
       </c>
       <c r="I122" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J122" s="5" t="n">
         <v>-0.03023857485534916</v>
@@ -8809,7 +9569,7 @@
         <v>-0.05660377358490566</v>
       </c>
       <c r="I124" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J124" s="5" t="n">
         <v>-0.056371434312831</v>
@@ -8881,7 +9641,7 @@
         <v>-0.8888574537540805</v>
       </c>
       <c r="I126" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J126" s="5" t="n">
         <v>-0.8886251144820059</v>
@@ -8953,7 +9713,7 @@
         <v>-0.007407407407407408</v>
       </c>
       <c r="I128" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J128" s="5" t="n">
         <v>-0.00717506813533274</v>
@@ -9025,7 +9785,7 @@
         <v>-0.08270676691729323</v>
       </c>
       <c r="I130" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J130" s="5" t="n">
         <v>-0.08247442764521856</v>
@@ -9097,7 +9857,7 @@
         <v>-0.01931818181818182</v>
       </c>
       <c r="I132" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J132" s="5" t="n">
         <v>-0.01908584254610715</v>
@@ -9169,7 +9929,7 @@
         <v>-0.05051813471502591</v>
       </c>
       <c r="I134" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J134" s="5" t="n">
         <v>-0.05028579544295124</v>
@@ -9241,7 +10001,7 @@
         <v>-0.06640926640926641</v>
       </c>
       <c r="I136" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J136" s="5" t="n">
         <v>-0.06617692713719174</v>
@@ -9313,7 +10073,7 @@
         <v>-0.06374269005847953</v>
       </c>
       <c r="I138" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J138" s="5" t="n">
         <v>-0.06351035078640486</v>
@@ -9385,7 +10145,7 @@
         <v>-0.0218303946263644</v>
       </c>
       <c r="I140" s="5" t="n">
-        <v>-0.000232339272074667</v>
+        <v>-0.0002323392720746678</v>
       </c>
       <c r="J140" s="5" t="n">
         <v>-0.02159805535428973</v>
@@ -11598,7 +12358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14571,6 +15331,506 @@
       <c r="J101" s="4" t="n"/>
       <c r="K101" s="4" t="n"/>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>1879</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>新日本建設</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="n">
+        <v>2178</v>
+      </c>
+      <c r="E102" s="4" t="n"/>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
+      <c r="J102" s="4" t="n"/>
+      <c r="K102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="n">
+        <v>3695</v>
+      </c>
+      <c r="E103" s="4" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
+      <c r="J103" s="4" t="n"/>
+      <c r="K103" s="4" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="n">
+        <v>2205</v>
+      </c>
+      <c r="E104" s="4" t="n"/>
+      <c r="F104" s="4" t="n"/>
+      <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
+      <c r="I104" s="4" t="n"/>
+      <c r="J104" s="4" t="n"/>
+      <c r="K104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="n">
+        <v>452</v>
+      </c>
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
+      <c r="I105" s="4" t="n"/>
+      <c r="J105" s="4" t="n"/>
+      <c r="K105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="n">
+        <v>2350</v>
+      </c>
+      <c r="E106" s="4" t="n"/>
+      <c r="F106" s="4" t="n"/>
+      <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
+      <c r="I106" s="4" t="n"/>
+      <c r="J106" s="4" t="n"/>
+      <c r="K106" s="4" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="n">
+        <v>1658</v>
+      </c>
+      <c r="E107" s="4" t="n"/>
+      <c r="F107" s="4" t="n"/>
+      <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
+      <c r="I107" s="4" t="n"/>
+      <c r="J107" s="4" t="n"/>
+      <c r="K107" s="4" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="n">
+        <v>4860</v>
+      </c>
+      <c r="E108" s="4" t="n"/>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
+      <c r="I108" s="4" t="n"/>
+      <c r="J108" s="4" t="n"/>
+      <c r="K108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="n">
+        <v>1112.5</v>
+      </c>
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="4" t="n"/>
+      <c r="K109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="n">
+        <v>2585</v>
+      </c>
+      <c r="E110" s="4" t="n"/>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n"/>
+      <c r="I110" s="4" t="n"/>
+      <c r="J110" s="4" t="n"/>
+      <c r="K110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>4187</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>大阪有機化学工業</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="n">
+        <v>4340</v>
+      </c>
+      <c r="E111" s="4" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
+      <c r="I111" s="4" t="n"/>
+      <c r="J111" s="4" t="n"/>
+      <c r="K111" s="4" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="n">
+        <v>2512</v>
+      </c>
+      <c r="E112" s="4" t="n"/>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
+      <c r="I112" s="4" t="n"/>
+      <c r="J112" s="4" t="n"/>
+      <c r="K112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="n">
+        <v>2582</v>
+      </c>
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
+      <c r="J113" s="4" t="n"/>
+      <c r="K113" s="4" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="n">
+        <v>3389</v>
+      </c>
+      <c r="E114" s="4" t="n"/>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
+      <c r="J114" s="4" t="n"/>
+      <c r="K114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="n">
+        <v>702</v>
+      </c>
+      <c r="E115" s="4" t="n"/>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
+      <c r="I115" s="4" t="n"/>
+      <c r="J115" s="4" t="n"/>
+      <c r="K115" s="4" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="n">
+        <v>2704</v>
+      </c>
+      <c r="E116" s="4" t="n"/>
+      <c r="F116" s="4" t="n"/>
+      <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
+      <c r="I116" s="4" t="n"/>
+      <c r="J116" s="4" t="n"/>
+      <c r="K116" s="4" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="n">
+        <v>857</v>
+      </c>
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
+      <c r="I117" s="4" t="n"/>
+      <c r="J117" s="4" t="n"/>
+      <c r="K117" s="4" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E118" s="4" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n"/>
+      <c r="K118" s="4" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="n">
+        <v>1361</v>
+      </c>
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
+      <c r="J119" s="4" t="n"/>
+      <c r="K119" s="4" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E120" s="4" t="n"/>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
+      <c r="I120" s="4" t="n"/>
+      <c r="J120" s="4" t="n"/>
+      <c r="K120" s="4" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>8739</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>スパークス・グループ</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="n">
+        <v>2438</v>
+      </c>
+      <c r="E121" s="4" t="n"/>
+      <c r="F121" s="4" t="n"/>
+      <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
+      <c r="I121" s="4" t="n"/>
+      <c r="J121" s="4" t="n"/>
+      <c r="K121" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Performance check 2026-10-17 -> 2026-10-24
</commit_message>
<xml_diff>
--- a/output/tracking_sheet.xlsx
+++ b/output/tracking_sheet.xlsx
@@ -5080,7 +5080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12347,6 +12347,726 @@
         <v>0.01652654779260055</v>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>1879</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>新日本建設</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E202" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F202" s="4" t="n">
+        <v>2197</v>
+      </c>
+      <c r="G202" s="4" t="n">
+        <v>2178</v>
+      </c>
+      <c r="H202" s="5" t="n">
+        <v>-0.008648156577150659</v>
+      </c>
+      <c r="I202" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J202" s="5" t="n">
+        <v>0.01959648925830047</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>朝日工業社</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E203" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F203" s="4" t="n">
+        <v>3860</v>
+      </c>
+      <c r="G203" s="4" t="n">
+        <v>3695</v>
+      </c>
+      <c r="H203" s="5" t="n">
+        <v>-0.0427461139896373</v>
+      </c>
+      <c r="I203" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J203" s="5" t="n">
+        <v>-0.01450146815418618</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>2288</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>丸大食品</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E204" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F204" s="4" t="n">
+        <v>2180</v>
+      </c>
+      <c r="G204" s="4" t="n">
+        <v>2205</v>
+      </c>
+      <c r="H204" s="5" t="n">
+        <v>0.01146788990825688</v>
+      </c>
+      <c r="I204" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J204" s="5" t="n">
+        <v>0.03971253574370801</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>システナ</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E205" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F205" s="4" t="n">
+        <v>458</v>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>452</v>
+      </c>
+      <c r="H205" s="5" t="n">
+        <v>-0.01310043668122271</v>
+      </c>
+      <c r="I205" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J205" s="5" t="n">
+        <v>0.01514420915422842</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>3150</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>グリムス</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E206" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F206" s="4" t="n">
+        <v>2378</v>
+      </c>
+      <c r="G206" s="4" t="n">
+        <v>2350</v>
+      </c>
+      <c r="H206" s="5" t="n">
+        <v>-0.01177460050462574</v>
+      </c>
+      <c r="I206" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J206" s="5" t="n">
+        <v>0.01647004533082539</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>3635</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>コーエーテクモホールディングス</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E207" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F207" s="4" t="n">
+        <v>1682</v>
+      </c>
+      <c r="G207" s="4" t="n">
+        <v>1658</v>
+      </c>
+      <c r="H207" s="5" t="n">
+        <v>-0.01426872770511296</v>
+      </c>
+      <c r="I207" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J207" s="5" t="n">
+        <v>0.01397591813033816</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>3817</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>ＳＲＡホールディングス</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E208" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F208" s="4" t="n">
+        <v>4820</v>
+      </c>
+      <c r="G208" s="4" t="n">
+        <v>4860</v>
+      </c>
+      <c r="H208" s="5" t="n">
+        <v>0.008298755186721992</v>
+      </c>
+      <c r="I208" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J208" s="5" t="n">
+        <v>0.03654340102217311</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>3854</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>アイル</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E209" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F209" s="4" t="n">
+        <v>2227</v>
+      </c>
+      <c r="G209" s="4" t="n">
+        <v>2342</v>
+      </c>
+      <c r="H209" s="5" t="n">
+        <v>0.05163897620116749</v>
+      </c>
+      <c r="I209" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J209" s="5" t="n">
+        <v>0.07988362203661861</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>3923</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>ラクス</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E210" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F210" s="4" t="n">
+        <v>1162</v>
+      </c>
+      <c r="G210" s="4" t="n">
+        <v>1112.5</v>
+      </c>
+      <c r="H210" s="5" t="n">
+        <v>-0.04259896729776248</v>
+      </c>
+      <c r="I210" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J210" s="5" t="n">
+        <v>-0.01435432146231135</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>4028</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>石原産業</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E211" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F211" s="4" t="n">
+        <v>2717</v>
+      </c>
+      <c r="G211" s="4" t="n">
+        <v>2585</v>
+      </c>
+      <c r="H211" s="5" t="n">
+        <v>-0.048582995951417</v>
+      </c>
+      <c r="I211" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J211" s="5" t="n">
+        <v>-0.02033835011596588</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>4503</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>アステラス製薬</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E212" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F212" s="4" t="n">
+        <v>2418.5</v>
+      </c>
+      <c r="G212" s="4" t="n">
+        <v>2512</v>
+      </c>
+      <c r="H212" s="5" t="n">
+        <v>0.03866032664874922</v>
+      </c>
+      <c r="I212" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J212" s="5" t="n">
+        <v>0.06690497248420035</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>5195</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>バンドー化学</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E213" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F213" s="4" t="n">
+        <v>2613</v>
+      </c>
+      <c r="G213" s="4" t="n">
+        <v>2582</v>
+      </c>
+      <c r="H213" s="5" t="n">
+        <v>-0.01186375813241485</v>
+      </c>
+      <c r="I213" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J213" s="5" t="n">
+        <v>0.01638088770303628</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>5334</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>日本特殊陶業</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E214" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F214" s="4" t="n">
+        <v>3679</v>
+      </c>
+      <c r="G214" s="4" t="n">
+        <v>3389</v>
+      </c>
+      <c r="H214" s="5" t="n">
+        <v>-0.07882576787170427</v>
+      </c>
+      <c r="I214" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J214" s="5" t="n">
+        <v>-0.05058112203625315</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>6200</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>インソース</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E215" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F215" s="4" t="n">
+        <v>703</v>
+      </c>
+      <c r="G215" s="4" t="n">
+        <v>702</v>
+      </c>
+      <c r="H215" s="5" t="n">
+        <v>-0.001422475106685633</v>
+      </c>
+      <c r="I215" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J215" s="5" t="n">
+        <v>0.02682217072876549</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>6331</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>三菱化工機</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E216" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F216" s="4" t="n">
+        <v>2786</v>
+      </c>
+      <c r="G216" s="4" t="n">
+        <v>2704</v>
+      </c>
+      <c r="H216" s="5" t="n">
+        <v>-0.02943287867910983</v>
+      </c>
+      <c r="I216" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J216" s="5" t="n">
+        <v>-0.00118823284365871</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>6727</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>ワコム</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E217" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F217" s="4" t="n">
+        <v>854</v>
+      </c>
+      <c r="G217" s="4" t="n">
+        <v>857</v>
+      </c>
+      <c r="H217" s="5" t="n">
+        <v>0.00351288056206089</v>
+      </c>
+      <c r="I217" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J217" s="5" t="n">
+        <v>0.03175752639751201</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>6750</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>エレコム</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E218" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F218" s="4" t="n">
+        <v>2016</v>
+      </c>
+      <c r="G218" s="4" t="n">
+        <v>1994</v>
+      </c>
+      <c r="H218" s="5" t="n">
+        <v>-0.01091269841269841</v>
+      </c>
+      <c r="I218" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J218" s="5" t="n">
+        <v>0.01733194742275271</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>7236</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>ティラド</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E219" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F219" s="4" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G219" s="4" t="n">
+        <v>1361</v>
+      </c>
+      <c r="H219" s="5" t="n">
+        <v>-0.04825174825174825</v>
+      </c>
+      <c r="I219" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J219" s="5" t="n">
+        <v>-0.02000710241629713</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>7595</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>アルゴグラフィックス</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E220" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F220" s="4" t="n">
+        <v>1324</v>
+      </c>
+      <c r="G220" s="4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="H220" s="5" t="n">
+        <v>-0.01812688821752266</v>
+      </c>
+      <c r="I220" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J220" s="5" t="n">
+        <v>0.01011775761792846</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>8624</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>いちよし証券</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E221" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F221" s="4" t="n">
+        <v>1572</v>
+      </c>
+      <c r="G221" s="4" t="n">
+        <v>1524</v>
+      </c>
+      <c r="H221" s="5" t="n">
+        <v>-0.03053435114503817</v>
+      </c>
+      <c r="I221" s="5" t="n">
+        <v>-0.02824464583545112</v>
+      </c>
+      <c r="J221" s="5" t="n">
+        <v>-0.002289705309587043</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12358,7 +13078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12372,6 +13092,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12430,6 +13151,11 @@
           <t>2026-10-17</t>
         </is>
       </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -12465,6 +13191,7 @@
       </c>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -12500,6 +13227,7 @@
       </c>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -12535,6 +13263,7 @@
       </c>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -12570,6 +13299,7 @@
       </c>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -12605,6 +13335,7 @@
       </c>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -12640,6 +13371,7 @@
       </c>
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -12675,6 +13407,7 @@
       </c>
       <c r="J8" s="4" t="n"/>
       <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -12710,6 +13443,7 @@
       </c>
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -12745,6 +13479,7 @@
       </c>
       <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -12780,6 +13515,7 @@
       </c>
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -12815,6 +13551,7 @@
       </c>
       <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -12850,6 +13587,7 @@
       </c>
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -12885,6 +13623,7 @@
       </c>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -12920,6 +13659,7 @@
       </c>
       <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -12955,6 +13695,7 @@
       </c>
       <c r="J16" s="4" t="n"/>
       <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -12990,6 +13731,7 @@
       </c>
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -13025,6 +13767,7 @@
       </c>
       <c r="J18" s="4" t="n"/>
       <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -13060,6 +13803,7 @@
       </c>
       <c r="J19" s="4" t="n"/>
       <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -13095,6 +13839,7 @@
       </c>
       <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -13130,6 +13875,7 @@
       </c>
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -13159,6 +13905,7 @@
       </c>
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -13188,6 +13935,7 @@
       </c>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -13217,6 +13965,7 @@
       </c>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -13246,6 +13995,7 @@
       </c>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -13275,6 +14025,7 @@
       </c>
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -13304,6 +14055,7 @@
       </c>
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -13333,6 +14085,7 @@
       </c>
       <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -13362,6 +14115,7 @@
       </c>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
+      <c r="L29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -13391,6 +14145,7 @@
       </c>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="n"/>
+      <c r="L30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -13420,6 +14175,7 @@
       </c>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -13449,6 +14205,7 @@
       </c>
       <c r="J32" s="4" t="n"/>
       <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -13478,6 +14235,7 @@
       </c>
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="n"/>
+      <c r="L33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -13507,6 +14265,7 @@
       </c>
       <c r="J34" s="4" t="n"/>
       <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -13536,6 +14295,7 @@
       </c>
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -13565,6 +14325,7 @@
       </c>
       <c r="J36" s="4" t="n"/>
       <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -13594,6 +14355,7 @@
       </c>
       <c r="J37" s="4" t="n"/>
       <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -13623,6 +14385,7 @@
       </c>
       <c r="J38" s="4" t="n"/>
       <c r="K38" s="4" t="n"/>
+      <c r="L38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -13652,6 +14415,7 @@
       </c>
       <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
+      <c r="L39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -13681,6 +14445,7 @@
       </c>
       <c r="J40" s="4" t="n"/>
       <c r="K40" s="4" t="n"/>
+      <c r="L40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -13710,6 +14475,7 @@
       </c>
       <c r="J41" s="4" t="n"/>
       <c r="K41" s="4" t="n"/>
+      <c r="L41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -13739,6 +14505,7 @@
         <v>935</v>
       </c>
       <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -13768,6 +14535,7 @@
         <v>3845</v>
       </c>
       <c r="K43" s="4" t="n"/>
+      <c r="L43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -13797,6 +14565,7 @@
         <v>2157</v>
       </c>
       <c r="K44" s="4" t="n"/>
+      <c r="L44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -13826,6 +14595,7 @@
         <v>433</v>
       </c>
       <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -13855,6 +14625,7 @@
         <v>3415</v>
       </c>
       <c r="K46" s="4" t="n"/>
+      <c r="L46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -13884,6 +14655,7 @@
         <v>2389</v>
       </c>
       <c r="K47" s="4" t="n"/>
+      <c r="L47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -13913,6 +14685,7 @@
         <v>1637</v>
       </c>
       <c r="K48" s="4" t="n"/>
+      <c r="L48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -13942,6 +14715,7 @@
         <v>4745</v>
       </c>
       <c r="K49" s="4" t="n"/>
+      <c r="L49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -13971,6 +14745,7 @@
         <v>2133</v>
       </c>
       <c r="K50" s="4" t="n"/>
+      <c r="L50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -14000,6 +14775,7 @@
         <v>2814</v>
       </c>
       <c r="K51" s="4" t="n"/>
+      <c r="L51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -14029,6 +14805,7 @@
         <v>2247.5</v>
       </c>
       <c r="K52" s="4" t="n"/>
+      <c r="L52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -14058,6 +14835,7 @@
         <v>2485</v>
       </c>
       <c r="K53" s="4" t="n"/>
+      <c r="L53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -14087,6 +14865,7 @@
         <v>3828</v>
       </c>
       <c r="K54" s="4" t="n"/>
+      <c r="L54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -14116,6 +14895,7 @@
         <v>695</v>
       </c>
       <c r="K55" s="4" t="n"/>
+      <c r="L55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -14145,6 +14925,7 @@
         <v>2918</v>
       </c>
       <c r="K56" s="4" t="n"/>
+      <c r="L56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -14174,6 +14955,7 @@
         <v>1431</v>
       </c>
       <c r="K57" s="4" t="n"/>
+      <c r="L57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -14203,6 +14985,7 @@
         <v>1241</v>
       </c>
       <c r="K58" s="4" t="n"/>
+      <c r="L58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -14232,6 +15015,7 @@
         <v>12445</v>
       </c>
       <c r="K59" s="4" t="n"/>
+      <c r="L59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -14261,6 +15045,7 @@
         <v>1561</v>
       </c>
       <c r="K60" s="4" t="n"/>
+      <c r="L60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -14290,6 +15075,7 @@
         <v>1185</v>
       </c>
       <c r="K61" s="4" t="n"/>
+      <c r="L61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -14317,6 +15103,7 @@
       <c r="K62" s="4" t="n">
         <v>3860</v>
       </c>
+      <c r="L62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -14344,6 +15131,7 @@
       <c r="K63" s="4" t="n">
         <v>2180</v>
       </c>
+      <c r="L63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -14371,6 +15159,7 @@
       <c r="K64" s="4" t="n">
         <v>458</v>
       </c>
+      <c r="L64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -14398,6 +15187,7 @@
       <c r="K65" s="4" t="n">
         <v>2989</v>
       </c>
+      <c r="L65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -14425,6 +15215,7 @@
       <c r="K66" s="4" t="n">
         <v>2378</v>
       </c>
+      <c r="L66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -14452,6 +15243,7 @@
       <c r="K67" s="4" t="n">
         <v>1682</v>
       </c>
+      <c r="L67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -14479,6 +15271,7 @@
       <c r="K68" s="4" t="n">
         <v>4820</v>
       </c>
+      <c r="L68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -14506,6 +15299,7 @@
       <c r="K69" s="4" t="n">
         <v>2227</v>
       </c>
+      <c r="L69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -14533,6 +15327,7 @@
       <c r="K70" s="4" t="n">
         <v>1162</v>
       </c>
+      <c r="L70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -14560,6 +15355,7 @@
       <c r="K71" s="4" t="n">
         <v>1382</v>
       </c>
+      <c r="L71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -14587,6 +15383,7 @@
       <c r="K72" s="4" t="n">
         <v>2717</v>
       </c>
+      <c r="L72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -14614,6 +15411,7 @@
       <c r="K73" s="4" t="n">
         <v>2418.5</v>
       </c>
+      <c r="L73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -14641,6 +15439,7 @@
       <c r="K74" s="4" t="n">
         <v>2613</v>
       </c>
+      <c r="L74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -14668,6 +15467,7 @@
       <c r="K75" s="4" t="n">
         <v>3679</v>
       </c>
+      <c r="L75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -14695,6 +15495,7 @@
       <c r="K76" s="4" t="n">
         <v>703</v>
       </c>
+      <c r="L76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -14722,6 +15523,7 @@
       <c r="K77" s="4" t="n">
         <v>2786</v>
       </c>
+      <c r="L77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -14749,6 +15551,7 @@
       <c r="K78" s="4" t="n">
         <v>2016</v>
       </c>
+      <c r="L78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -14776,6 +15579,7 @@
       <c r="K79" s="4" t="n">
         <v>1430</v>
       </c>
+      <c r="L79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -14803,6 +15607,7 @@
       <c r="K80" s="4" t="n">
         <v>1324</v>
       </c>
+      <c r="L80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -14830,6 +15635,7 @@
       <c r="K81" s="4" t="n">
         <v>1572</v>
       </c>
+      <c r="L81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -14855,6 +15661,9 @@
       <c r="I82" s="4" t="n"/>
       <c r="J82" s="4" t="n"/>
       <c r="K82" s="4" t="n"/>
+      <c r="L82" s="4" t="n">
+        <v>2178</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -14880,6 +15689,9 @@
       <c r="I83" s="4" t="n"/>
       <c r="J83" s="4" t="n"/>
       <c r="K83" s="4" t="n"/>
+      <c r="L83" s="4" t="n">
+        <v>3695</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -14905,6 +15717,9 @@
       <c r="I84" s="4" t="n"/>
       <c r="J84" s="4" t="n"/>
       <c r="K84" s="4" t="n"/>
+      <c r="L84" s="4" t="n">
+        <v>2205</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -14930,6 +15745,9 @@
       <c r="I85" s="4" t="n"/>
       <c r="J85" s="4" t="n"/>
       <c r="K85" s="4" t="n"/>
+      <c r="L85" s="4" t="n">
+        <v>452</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -14955,6 +15773,9 @@
       <c r="I86" s="4" t="n"/>
       <c r="J86" s="4" t="n"/>
       <c r="K86" s="4" t="n"/>
+      <c r="L86" s="4" t="n">
+        <v>2350</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -14980,6 +15801,9 @@
       <c r="I87" s="4" t="n"/>
       <c r="J87" s="4" t="n"/>
       <c r="K87" s="4" t="n"/>
+      <c r="L87" s="4" t="n">
+        <v>1658</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -15005,6 +15829,9 @@
       <c r="I88" s="4" t="n"/>
       <c r="J88" s="4" t="n"/>
       <c r="K88" s="4" t="n"/>
+      <c r="L88" s="4" t="n">
+        <v>4860</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -15030,6 +15857,9 @@
       <c r="I89" s="4" t="n"/>
       <c r="J89" s="4" t="n"/>
       <c r="K89" s="4" t="n"/>
+      <c r="L89" s="4" t="n">
+        <v>2342</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -15055,6 +15885,9 @@
       <c r="I90" s="4" t="n"/>
       <c r="J90" s="4" t="n"/>
       <c r="K90" s="4" t="n"/>
+      <c r="L90" s="4" t="n">
+        <v>1112.5</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -15080,6 +15913,9 @@
       <c r="I91" s="4" t="n"/>
       <c r="J91" s="4" t="n"/>
       <c r="K91" s="4" t="n"/>
+      <c r="L91" s="4" t="n">
+        <v>2585</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -15105,6 +15941,9 @@
       <c r="I92" s="4" t="n"/>
       <c r="J92" s="4" t="n"/>
       <c r="K92" s="4" t="n"/>
+      <c r="L92" s="4" t="n">
+        <v>2512</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -15130,6 +15969,9 @@
       <c r="I93" s="4" t="n"/>
       <c r="J93" s="4" t="n"/>
       <c r="K93" s="4" t="n"/>
+      <c r="L93" s="4" t="n">
+        <v>2582</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -15155,6 +15997,9 @@
       <c r="I94" s="4" t="n"/>
       <c r="J94" s="4" t="n"/>
       <c r="K94" s="4" t="n"/>
+      <c r="L94" s="4" t="n">
+        <v>3389</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -15180,6 +16025,9 @@
       <c r="I95" s="4" t="n"/>
       <c r="J95" s="4" t="n"/>
       <c r="K95" s="4" t="n"/>
+      <c r="L95" s="4" t="n">
+        <v>702</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -15205,6 +16053,9 @@
       <c r="I96" s="4" t="n"/>
       <c r="J96" s="4" t="n"/>
       <c r="K96" s="4" t="n"/>
+      <c r="L96" s="4" t="n">
+        <v>2704</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -15230,6 +16081,9 @@
       <c r="I97" s="4" t="n"/>
       <c r="J97" s="4" t="n"/>
       <c r="K97" s="4" t="n"/>
+      <c r="L97" s="4" t="n">
+        <v>857</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -15255,6 +16109,9 @@
       <c r="I98" s="4" t="n"/>
       <c r="J98" s="4" t="n"/>
       <c r="K98" s="4" t="n"/>
+      <c r="L98" s="4" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -15280,6 +16137,9 @@
       <c r="I99" s="4" t="n"/>
       <c r="J99" s="4" t="n"/>
       <c r="K99" s="4" t="n"/>
+      <c r="L99" s="4" t="n">
+        <v>1361</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -15305,6 +16165,9 @@
       <c r="I100" s="4" t="n"/>
       <c r="J100" s="4" t="n"/>
       <c r="K100" s="4" t="n"/>
+      <c r="L100" s="4" t="n">
+        <v>1300</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -15330,6 +16193,9 @@
       <c r="I101" s="4" t="n"/>
       <c r="J101" s="4" t="n"/>
       <c r="K101" s="4" t="n"/>
+      <c r="L101" s="4" t="n">
+        <v>1524</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -15355,6 +16221,7 @@
       <c r="I102" s="4" t="n"/>
       <c r="J102" s="4" t="n"/>
       <c r="K102" s="4" t="n"/>
+      <c r="L102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -15380,6 +16247,7 @@
       <c r="I103" s="4" t="n"/>
       <c r="J103" s="4" t="n"/>
       <c r="K103" s="4" t="n"/>
+      <c r="L103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -15405,6 +16273,7 @@
       <c r="I104" s="4" t="n"/>
       <c r="J104" s="4" t="n"/>
       <c r="K104" s="4" t="n"/>
+      <c r="L104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -15430,6 +16299,7 @@
       <c r="I105" s="4" t="n"/>
       <c r="J105" s="4" t="n"/>
       <c r="K105" s="4" t="n"/>
+      <c r="L105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -15455,6 +16325,7 @@
       <c r="I106" s="4" t="n"/>
       <c r="J106" s="4" t="n"/>
       <c r="K106" s="4" t="n"/>
+      <c r="L106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -15480,6 +16351,7 @@
       <c r="I107" s="4" t="n"/>
       <c r="J107" s="4" t="n"/>
       <c r="K107" s="4" t="n"/>
+      <c r="L107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -15505,6 +16377,7 @@
       <c r="I108" s="4" t="n"/>
       <c r="J108" s="4" t="n"/>
       <c r="K108" s="4" t="n"/>
+      <c r="L108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -15530,6 +16403,7 @@
       <c r="I109" s="4" t="n"/>
       <c r="J109" s="4" t="n"/>
       <c r="K109" s="4" t="n"/>
+      <c r="L109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -15555,6 +16429,7 @@
       <c r="I110" s="4" t="n"/>
       <c r="J110" s="4" t="n"/>
       <c r="K110" s="4" t="n"/>
+      <c r="L110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -15580,6 +16455,7 @@
       <c r="I111" s="4" t="n"/>
       <c r="J111" s="4" t="n"/>
       <c r="K111" s="4" t="n"/>
+      <c r="L111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -15605,6 +16481,7 @@
       <c r="I112" s="4" t="n"/>
       <c r="J112" s="4" t="n"/>
       <c r="K112" s="4" t="n"/>
+      <c r="L112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -15630,6 +16507,7 @@
       <c r="I113" s="4" t="n"/>
       <c r="J113" s="4" t="n"/>
       <c r="K113" s="4" t="n"/>
+      <c r="L113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -15655,6 +16533,7 @@
       <c r="I114" s="4" t="n"/>
       <c r="J114" s="4" t="n"/>
       <c r="K114" s="4" t="n"/>
+      <c r="L114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -15680,6 +16559,7 @@
       <c r="I115" s="4" t="n"/>
       <c r="J115" s="4" t="n"/>
       <c r="K115" s="4" t="n"/>
+      <c r="L115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -15705,6 +16585,7 @@
       <c r="I116" s="4" t="n"/>
       <c r="J116" s="4" t="n"/>
       <c r="K116" s="4" t="n"/>
+      <c r="L116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -15730,6 +16611,7 @@
       <c r="I117" s="4" t="n"/>
       <c r="J117" s="4" t="n"/>
       <c r="K117" s="4" t="n"/>
+      <c r="L117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -15755,6 +16637,7 @@
       <c r="I118" s="4" t="n"/>
       <c r="J118" s="4" t="n"/>
       <c r="K118" s="4" t="n"/>
+      <c r="L118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -15780,6 +16663,7 @@
       <c r="I119" s="4" t="n"/>
       <c r="J119" s="4" t="n"/>
       <c r="K119" s="4" t="n"/>
+      <c r="L119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -15805,6 +16689,7 @@
       <c r="I120" s="4" t="n"/>
       <c r="J120" s="4" t="n"/>
       <c r="K120" s="4" t="n"/>
+      <c r="L120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -15830,6 +16715,7 @@
       <c r="I121" s="4" t="n"/>
       <c r="J121" s="4" t="n"/>
       <c r="K121" s="4" t="n"/>
+      <c r="L121" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>